<commit_message>
Build all teaching workbooks with desktop Excel
</commit_message>
<xml_diff>
--- a/data/kapitola_05.xlsx
+++ b/data/kapitola_05.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="202300"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{7CAF77E1-AE13-4CB7-BA51-807534603A2E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{E68C876B-4860-4929-9365-53A085875B78}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-109" yWindow="-109" windowWidth="34995" windowHeight="19060" xr2:uid="{1CF803C7-E1EE-4F21-98EB-C4BFD4F9078C}"/>
+    <workbookView xWindow="-109" yWindow="-109" windowWidth="34995" windowHeight="19060" xr2:uid="{DE02CC22-A075-4BAC-A50D-3760BFE17441}"/>
   </bookViews>
   <sheets>
     <sheet name="Prehled" sheetId="1" r:id="rId1"/>
@@ -273,6 +273,9 @@
     <t>Slovní druh</t>
   </si>
   <si>
+    <t>Počet kartiček</t>
+  </si>
+  <si>
     <t>Podstatné jméno</t>
   </si>
   <si>
@@ -282,9 +285,6 @@
     <t>Přídavné jméno</t>
   </si>
   <si>
-    <t>Počet kartiček</t>
-  </si>
-  <si>
     <t>Použití a původ</t>
   </si>
   <si>
@@ -297,18 +297,18 @@
     <t>Pohlaví</t>
   </si>
   <si>
+    <t>Stres</t>
+  </si>
+  <si>
+    <t>Pohoda</t>
+  </si>
+  <si>
     <t>Žena</t>
   </si>
   <si>
     <t>Muž</t>
   </si>
   <si>
-    <t>Stres</t>
-  </si>
-  <si>
-    <t>Pohoda</t>
-  </si>
-  <si>
     <t>Výklad: průnik, sjednocení, podmíněná pravděpodobnost, závislost</t>
   </si>
   <si>
@@ -396,6 +396,9 @@
     <t>Emoce</t>
   </si>
   <si>
+    <t>Počet fotografií</t>
+  </si>
+  <si>
     <t>Radost</t>
   </si>
   <si>
@@ -408,9 +411,6 @@
     <t>Překvapení</t>
   </si>
   <si>
-    <t>Počet fotografií</t>
-  </si>
-  <si>
     <t>Cvičení 1</t>
   </si>
   <si>
@@ -420,18 +420,18 @@
     <t>Sport</t>
   </si>
   <si>
+    <t>Dobrý spánek</t>
+  </si>
+  <si>
+    <t>Špatný spánek</t>
+  </si>
+  <si>
     <t>Sportuje</t>
   </si>
   <si>
     <t>Nesportuje</t>
   </si>
   <si>
-    <t>Dobrý spánek</t>
-  </si>
-  <si>
-    <t>Špatný spánek</t>
-  </si>
-  <si>
     <t>Cvičení 3</t>
   </si>
   <si>
@@ -522,127 +522,127 @@
     <t>Zadání a vysvětlení jsou v kapitole. Řešení otevírejte až po vlastním pokusu.</t>
   </si>
   <si>
+    <t>List</t>
+  </si>
+  <si>
+    <t>Oblast vstupů / tabulky</t>
+  </si>
+  <si>
+    <t>Příklad nebo cvičení</t>
+  </si>
+  <si>
+    <t>Karticky</t>
+  </si>
+  <si>
+    <t>A2:B4</t>
+  </si>
+  <si>
+    <t>Tabulka_zavislost</t>
+  </si>
+  <si>
+    <t>A2:C3</t>
+  </si>
+  <si>
+    <t>Tabulka_nezavislost</t>
+  </si>
+  <si>
+    <t>A2:B7</t>
+  </si>
+  <si>
+    <t>Test_hadani</t>
+  </si>
+  <si>
+    <t>Sim_hadani</t>
+  </si>
+  <si>
+    <t>A2:A41</t>
+  </si>
+  <si>
+    <t>Rozpoznavani</t>
+  </si>
+  <si>
+    <t>Losovani</t>
+  </si>
+  <si>
+    <t>A2:B3</t>
+  </si>
+  <si>
+    <t>U01_emoce</t>
+  </si>
+  <si>
+    <t>A2:B5</t>
+  </si>
+  <si>
+    <t>U03_tabulka</t>
+  </si>
+  <si>
+    <t>U04_vstupy</t>
+  </si>
+  <si>
+    <t>U06_screening</t>
+  </si>
+  <si>
+    <t>A2:B6</t>
+  </si>
+  <si>
+    <t>U07_taxi</t>
+  </si>
+  <si>
+    <t>U08_rozdeleni</t>
+  </si>
+  <si>
+    <t>A2:C5</t>
+  </si>
+  <si>
+    <t>U09_test</t>
+  </si>
+  <si>
+    <t>U10_test</t>
+  </si>
+  <si>
+    <t>U11_aproximace</t>
+  </si>
+  <si>
+    <t>Bayes</t>
+  </si>
+  <si>
+    <t>A1:B20</t>
+  </si>
+  <si>
+    <t>Hotové přirozené četnosti, úplná pravděpodobnost a Bayesova věta</t>
+  </si>
+  <si>
+    <t>Binom</t>
+  </si>
+  <si>
+    <t>A1:D19</t>
+  </si>
+  <si>
+    <t>Hotové binomické rozdělení pro pět otázek</t>
+  </si>
+  <si>
+    <t>Binom_20</t>
+  </si>
+  <si>
+    <t>A1:E22</t>
+  </si>
+  <si>
+    <t>Hotové výpočty právě, nejvýše a alespoň pro dvacet otázek</t>
+  </si>
+  <si>
+    <t>Aproximace</t>
+  </si>
+  <si>
+    <t>A1:B16</t>
+  </si>
+  <si>
+    <t>Hotová normální aproximace, přesná hodnota a převod na podíl</t>
+  </si>
+  <si>
     <t>Slovní úlohy bez konkrétních čísel nevyžadují vlastní datový list.</t>
   </si>
   <si>
     <t>Pravděpodobnosti a modelové četnosti nejsou záznamy o jednotlivých lidech.</t>
-  </si>
-  <si>
-    <t>List</t>
-  </si>
-  <si>
-    <t>Oblast vstupů / tabulky</t>
-  </si>
-  <si>
-    <t>Příklad nebo cvičení</t>
-  </si>
-  <si>
-    <t>Karticky</t>
-  </si>
-  <si>
-    <t>A2:B4</t>
-  </si>
-  <si>
-    <t>Tabulka_zavislost</t>
-  </si>
-  <si>
-    <t>A2:C3</t>
-  </si>
-  <si>
-    <t>Tabulka_nezavislost</t>
-  </si>
-  <si>
-    <t>A2:B7</t>
-  </si>
-  <si>
-    <t>Test_hadani</t>
-  </si>
-  <si>
-    <t>Sim_hadani</t>
-  </si>
-  <si>
-    <t>A2:A41</t>
-  </si>
-  <si>
-    <t>Rozpoznavani</t>
-  </si>
-  <si>
-    <t>Losovani</t>
-  </si>
-  <si>
-    <t>A2:B3</t>
-  </si>
-  <si>
-    <t>U01_emoce</t>
-  </si>
-  <si>
-    <t>A2:B5</t>
-  </si>
-  <si>
-    <t>U03_tabulka</t>
-  </si>
-  <si>
-    <t>U04_vstupy</t>
-  </si>
-  <si>
-    <t>U06_screening</t>
-  </si>
-  <si>
-    <t>A2:B6</t>
-  </si>
-  <si>
-    <t>U07_taxi</t>
-  </si>
-  <si>
-    <t>U08_rozdeleni</t>
-  </si>
-  <si>
-    <t>A2:C5</t>
-  </si>
-  <si>
-    <t>U09_test</t>
-  </si>
-  <si>
-    <t>U10_test</t>
-  </si>
-  <si>
-    <t>U11_aproximace</t>
-  </si>
-  <si>
-    <t>Bayes</t>
-  </si>
-  <si>
-    <t>A1:B20</t>
-  </si>
-  <si>
-    <t>Hotové přirozené četnosti, úplná pravděpodobnost a Bayesova věta</t>
-  </si>
-  <si>
-    <t>Binom</t>
-  </si>
-  <si>
-    <t>A1:D19</t>
-  </si>
-  <si>
-    <t>Hotové binomické rozdělení pro pět otázek</t>
-  </si>
-  <si>
-    <t>Binom_20</t>
-  </si>
-  <si>
-    <t>A1:E22</t>
-  </si>
-  <si>
-    <t>Hotové výpočty právě, nejvýše a alespoň pro dvacet otázek</t>
-  </si>
-  <si>
-    <t>Aproximace</t>
-  </si>
-  <si>
-    <t>A1:B16</t>
-  </si>
-  <si>
-    <t>Hotová normální aproximace, přesná hodnota a převod na podíl</t>
   </si>
 </sst>
 </file>
@@ -732,12 +732,18 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="3" fontId="1" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
@@ -752,7 +758,7 @@
     <xf numFmtId="164" fontId="1" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="1" fontId="1" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
@@ -773,16 +779,22 @@
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -1118,7 +1130,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{29DC03EB-420D-4784-A377-1655B3043EE5}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D0F6EF17-C69F-477C-AE36-E3352F7C5F8B}">
   <dimension ref="A1:C31"/>
   <sheetFormatPr defaultRowHeight="14.3" x14ac:dyDescent="0.25"/>
   <cols>
@@ -1127,11 +1139,11 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" ht="30.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="17" t="s">
+      <c r="A1" s="21" t="s">
         <v>152</v>
       </c>
-      <c r="B1" s="16"/>
-      <c r="C1" s="16"/>
+      <c r="B1" s="19"/>
+      <c r="C1" s="19"/>
     </row>
     <row r="2" spans="1:3" ht="30.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="1"/>
@@ -1139,273 +1151,273 @@
       <c r="C2" s="1"/>
     </row>
     <row r="3" spans="1:3" ht="30.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="16" t="s">
+      <c r="A3" s="20" t="s">
         <v>153</v>
       </c>
-      <c r="B3" s="16"/>
-      <c r="C3" s="16"/>
+      <c r="B3" s="19"/>
+      <c r="C3" s="19"/>
     </row>
     <row r="4" spans="1:3" ht="30.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="16" t="s">
+      <c r="A4" s="20" t="s">
         <v>154</v>
       </c>
-      <c r="B4" s="16"/>
-      <c r="C4" s="16"/>
+      <c r="B4" s="19"/>
+      <c r="C4" s="19"/>
     </row>
     <row r="5" spans="1:3" ht="30.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="16" t="s">
+      <c r="A5" s="20" t="s">
+        <v>194</v>
+      </c>
+      <c r="B5" s="19"/>
+      <c r="C5" s="19"/>
+    </row>
+    <row r="6" spans="1:3" ht="30.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="20" t="s">
+        <v>195</v>
+      </c>
+      <c r="B6" s="19"/>
+      <c r="C6" s="19"/>
+    </row>
+    <row r="7" spans="1:3" ht="30.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="3" t="s">
         <v>155</v>
       </c>
-      <c r="B5" s="16"/>
-      <c r="C5" s="16"/>
-    </row>
-    <row r="6" spans="1:3" ht="30.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="16" t="s">
+      <c r="B7" s="3" t="s">
         <v>156</v>
       </c>
-      <c r="B6" s="16"/>
-      <c r="C6" s="16"/>
-    </row>
-    <row r="7" spans="1:3" ht="30.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="2" t="s">
+      <c r="C7" s="3" t="s">
         <v>157</v>
       </c>
-      <c r="B7" s="2" t="s">
+    </row>
+    <row r="8" spans="1:3" ht="30.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="2" t="s">
         <v>158</v>
       </c>
-      <c r="C7" s="2" t="s">
+      <c r="B8" s="2" t="s">
         <v>159</v>
       </c>
-    </row>
-    <row r="8" spans="1:3" ht="30.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="1" t="s">
+      <c r="C8" s="2" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" ht="30.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="2" t="s">
         <v>160</v>
       </c>
-      <c r="B8" s="1" t="s">
+      <c r="B9" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="C8" s="1" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" ht="30.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="1" t="s">
+      <c r="C9" s="2" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" ht="30.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="2" t="s">
         <v>162</v>
       </c>
-      <c r="B9" s="1" t="s">
+      <c r="B10" s="2" t="s">
+        <v>161</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" ht="30.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B11" s="2" t="s">
         <v>163</v>
       </c>
-      <c r="C9" s="1" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" ht="30.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="1" t="s">
+      <c r="C11" s="2" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" ht="30.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="2" t="s">
         <v>164</v>
       </c>
-      <c r="B10" s="1" t="s">
+      <c r="B12" s="2" t="s">
         <v>163</v>
       </c>
-      <c r="C10" s="1" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" ht="30.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B11" s="1" t="s">
+      <c r="C12" s="2" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" ht="30.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="2" t="s">
         <v>165</v>
       </c>
-      <c r="C11" s="1" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" ht="30.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="1" t="s">
+      <c r="B13" s="2" t="s">
         <v>166</v>
       </c>
-      <c r="B12" s="1" t="s">
-        <v>165</v>
-      </c>
-      <c r="C12" s="1" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3" ht="30.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="1" t="s">
+      <c r="C13" s="2" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" ht="30.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="2" t="s">
         <v>167</v>
       </c>
-      <c r="B13" s="1" t="s">
+      <c r="B14" s="2" t="s">
+        <v>159</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" ht="30.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="2" t="s">
         <v>168</v>
       </c>
-      <c r="C13" s="1" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3" ht="30.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="1" t="s">
+      <c r="B15" s="2" t="s">
         <v>169</v>
       </c>
-      <c r="B14" s="1" t="s">
+      <c r="C15" s="2" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" ht="30.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="2" t="s">
+        <v>170</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>171</v>
+      </c>
+      <c r="C16" s="2" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" ht="30.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="2" t="s">
+        <v>172</v>
+      </c>
+      <c r="B17" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="C14" s="1" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="15" spans="1:3" ht="30.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="1" t="s">
-        <v>170</v>
-      </c>
-      <c r="B15" s="1" t="s">
+      <c r="C17" s="2" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" ht="30.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="2" t="s">
+        <v>173</v>
+      </c>
+      <c r="B18" s="2" t="s">
         <v>171</v>
       </c>
-      <c r="C15" s="1" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="16" spans="1:3" ht="30.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="1" t="s">
-        <v>172</v>
-      </c>
-      <c r="B16" s="1" t="s">
-        <v>173</v>
-      </c>
-      <c r="C16" s="1" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="17" spans="1:3" ht="30.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="1" t="s">
+      <c r="C18" s="2" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" ht="30.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="2" t="s">
         <v>174</v>
       </c>
-      <c r="B17" s="1" t="s">
-        <v>163</v>
-      </c>
-      <c r="C17" s="1" t="s">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="18" spans="1:3" ht="30.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="1" t="s">
+      <c r="B19" s="2" t="s">
         <v>175</v>
       </c>
-      <c r="B18" s="1" t="s">
-        <v>173</v>
-      </c>
-      <c r="C18" s="1" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="19" spans="1:3" ht="30.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="1" t="s">
+      <c r="C19" s="2" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" ht="30.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="2" t="s">
         <v>176</v>
       </c>
-      <c r="B19" s="1" t="s">
+      <c r="B20" s="2" t="s">
+        <v>159</v>
+      </c>
+      <c r="C20" s="2" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" ht="30.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="2" t="s">
         <v>177</v>
       </c>
-      <c r="C19" s="1" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="20" spans="1:3" ht="30.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="1" t="s">
+      <c r="B21" s="2" t="s">
         <v>178</v>
       </c>
-      <c r="B20" s="1" t="s">
-        <v>161</v>
-      </c>
-      <c r="C20" s="1" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="21" spans="1:3" ht="30.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="1" t="s">
+      <c r="C21" s="2" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" ht="30.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="2" t="s">
         <v>179</v>
       </c>
-      <c r="B21" s="1" t="s">
+      <c r="B22" s="2" t="s">
+        <v>159</v>
+      </c>
+      <c r="C22" s="2" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" ht="30.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A23" s="2" t="s">
         <v>180</v>
       </c>
-      <c r="C21" s="1" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="22" spans="1:3" ht="30.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="1" t="s">
+      <c r="B23" s="2" t="s">
+        <v>171</v>
+      </c>
+      <c r="C23" s="2" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" ht="30.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="2" t="s">
         <v>181</v>
       </c>
-      <c r="B22" s="1" t="s">
-        <v>161</v>
-      </c>
-      <c r="C22" s="1" t="s">
-        <v>148</v>
-      </c>
-    </row>
-    <row r="23" spans="1:3" ht="30.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="1" t="s">
+      <c r="B24" s="2" t="s">
+        <v>159</v>
+      </c>
+      <c r="C24" s="2" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" ht="30.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A25" s="2" t="s">
         <v>182</v>
       </c>
-      <c r="B23" s="1" t="s">
-        <v>173</v>
-      </c>
-      <c r="C23" s="1" t="s">
-        <v>149</v>
-      </c>
-    </row>
-    <row r="24" spans="1:3" ht="30.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="1" t="s">
+      <c r="B25" s="2" t="s">
         <v>183</v>
       </c>
-      <c r="B24" s="1" t="s">
-        <v>161</v>
-      </c>
-      <c r="C24" s="1" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="25" spans="1:3" ht="30.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="1" t="s">
+      <c r="C25" s="2" t="s">
         <v>184</v>
       </c>
-      <c r="B25" s="1" t="s">
+    </row>
+    <row r="26" spans="1:3" ht="30.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A26" s="2" t="s">
         <v>185</v>
       </c>
-      <c r="C25" s="1" t="s">
+      <c r="B26" s="2" t="s">
         <v>186</v>
       </c>
-    </row>
-    <row r="26" spans="1:3" ht="30.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="1" t="s">
+      <c r="C26" s="2" t="s">
         <v>187</v>
       </c>
-      <c r="B26" s="1" t="s">
+    </row>
+    <row r="27" spans="1:3" ht="30.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A27" s="2" t="s">
         <v>188</v>
       </c>
-      <c r="C26" s="1" t="s">
+      <c r="B27" s="2" t="s">
         <v>189</v>
       </c>
-    </row>
-    <row r="27" spans="1:3" ht="30.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="1" t="s">
+      <c r="C27" s="2" t="s">
         <v>190</v>
       </c>
-      <c r="B27" s="1" t="s">
+    </row>
+    <row r="28" spans="1:3" ht="30.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A28" s="2" t="s">
         <v>191</v>
       </c>
-      <c r="C27" s="1" t="s">
+      <c r="B28" s="2" t="s">
         <v>192</v>
       </c>
-    </row>
-    <row r="28" spans="1:3" ht="30.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="1" t="s">
+      <c r="C28" s="2" t="s">
         <v>193</v>
-      </c>
-      <c r="B28" s="1" t="s">
-        <v>194</v>
-      </c>
-      <c r="C28" s="1" t="s">
-        <v>195</v>
       </c>
     </row>
     <row r="29" spans="1:3" ht="30.1" customHeight="1" x14ac:dyDescent="0.25">
@@ -1436,7 +1448,7 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C786966A-DC9E-4224-8E0D-C4F8DB62CD84}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9E327118-9EA2-41A7-9E8C-7332AE1B9E00}">
   <dimension ref="A1:D7"/>
   <sheetFormatPr defaultRowHeight="14.3" x14ac:dyDescent="0.25"/>
   <cols>
@@ -1446,73 +1458,73 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="46.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="4" t="s">
         <v>88</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="14" t="s">
+      <c r="D1" s="16" t="s">
         <v>76</v>
       </c>
     </row>
     <row r="2" spans="1:4" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="13" t="s">
+      <c r="A2" s="15" t="s">
         <v>94</v>
       </c>
-      <c r="B2" s="13">
+      <c r="B2" s="15">
         <v>5</v>
       </c>
-      <c r="D2" s="15" t="s">
+      <c r="D2" s="18" t="s">
         <v>98</v>
       </c>
     </row>
     <row r="3" spans="1:4" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="13" t="s">
+      <c r="A3" s="15" t="s">
         <v>95</v>
       </c>
-      <c r="B3" s="13">
+      <c r="B3" s="15">
         <v>4</v>
       </c>
-      <c r="D3" s="15"/>
+      <c r="D3" s="17"/>
     </row>
     <row r="4" spans="1:4" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="13" t="s">
+      <c r="A4" s="15" t="s">
         <v>96</v>
       </c>
-      <c r="B4" s="13">
+      <c r="B4" s="15">
         <v>0.25</v>
       </c>
-      <c r="D4" s="15" t="s">
+      <c r="D4" s="18" t="s">
         <v>99</v>
       </c>
     </row>
     <row r="5" spans="1:4" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="13" t="s">
+      <c r="A5" s="15" t="s">
         <v>97</v>
       </c>
-      <c r="B5" s="13">
+      <c r="B5" s="15">
         <v>20</v>
       </c>
-      <c r="D5" s="15"/>
+      <c r="D5" s="17"/>
     </row>
     <row r="6" spans="1:4" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="13" t="s">
+      <c r="A6" s="15" t="s">
         <v>46</v>
       </c>
-      <c r="B6" s="13">
+      <c r="B6" s="15">
         <v>5</v>
       </c>
-      <c r="D6" s="15"/>
+      <c r="D6" s="17"/>
     </row>
     <row r="7" spans="1:4" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="13" t="s">
+      <c r="A7" s="15" t="s">
         <v>47</v>
       </c>
-      <c r="B7" s="13">
+      <c r="B7" s="15">
         <v>10</v>
       </c>
-      <c r="D7" s="15"/>
+      <c r="D7" s="17"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -1524,7 +1536,7 @@
 </file>
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{43B61429-9CF2-49DB-899B-58B549D88B2A}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B49852BA-8822-4B9A-AA77-38F63278489B}">
   <dimension ref="A1:C41"/>
   <sheetFormatPr defaultRowHeight="14.3" x14ac:dyDescent="0.25"/>
   <cols>
@@ -1533,220 +1545,220 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" ht="46.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="4" t="s">
         <v>100</v>
       </c>
-      <c r="C1" s="14" t="s">
+      <c r="C1" s="16" t="s">
         <v>76</v>
       </c>
     </row>
     <row r="2" spans="1:3" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="13">
+      <c r="A2" s="15">
         <v>2</v>
       </c>
-      <c r="C2" s="15" t="s">
+      <c r="C2" s="18" t="s">
         <v>101</v>
       </c>
     </row>
     <row r="3" spans="1:3" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="13">
+      <c r="A3" s="15">
         <v>1</v>
       </c>
-      <c r="C3" s="15"/>
+      <c r="C3" s="17"/>
     </row>
     <row r="4" spans="1:3" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="13">
+      <c r="A4" s="15">
         <v>2</v>
       </c>
-      <c r="C4" s="15" t="s">
+      <c r="C4" s="18" t="s">
         <v>102</v>
       </c>
     </row>
     <row r="5" spans="1:3" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="13">
+      <c r="A5" s="15">
         <v>3</v>
       </c>
-      <c r="C5" s="15"/>
+      <c r="C5" s="17"/>
     </row>
     <row r="6" spans="1:3" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="13">
+      <c r="A6" s="15">
         <v>1</v>
       </c>
-      <c r="C6" s="15"/>
+      <c r="C6" s="17"/>
     </row>
     <row r="7" spans="1:3" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="13">
+      <c r="A7" s="15">
         <v>0</v>
       </c>
-      <c r="C7" s="15"/>
+      <c r="C7" s="17"/>
     </row>
     <row r="8" spans="1:3" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="13">
+      <c r="A8" s="15">
         <v>2</v>
       </c>
     </row>
     <row r="9" spans="1:3" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="13">
+      <c r="A9" s="15">
         <v>2</v>
       </c>
     </row>
     <row r="10" spans="1:3" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="13">
+      <c r="A10" s="15">
         <v>1</v>
       </c>
     </row>
     <row r="11" spans="1:3" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="13">
+      <c r="A11" s="15">
         <v>2</v>
       </c>
     </row>
     <row r="12" spans="1:3" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="13">
+      <c r="A12" s="15">
         <v>1</v>
       </c>
     </row>
     <row r="13" spans="1:3" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="13">
+      <c r="A13" s="15">
         <v>0</v>
       </c>
     </row>
     <row r="14" spans="1:3" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="13">
+      <c r="A14" s="15">
         <v>0</v>
       </c>
     </row>
     <row r="15" spans="1:3" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="13">
+      <c r="A15" s="15">
         <v>1</v>
       </c>
     </row>
     <row r="16" spans="1:3" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="13">
+      <c r="A16" s="15">
         <v>2</v>
       </c>
     </row>
     <row r="17" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="13">
+      <c r="A17" s="15">
         <v>0</v>
       </c>
     </row>
     <row r="18" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="13">
+      <c r="A18" s="15">
         <v>0</v>
       </c>
     </row>
     <row r="19" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="13">
+      <c r="A19" s="15">
         <v>1</v>
       </c>
     </row>
     <row r="20" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="13">
+      <c r="A20" s="15">
         <v>1</v>
       </c>
     </row>
     <row r="21" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="13">
+      <c r="A21" s="15">
         <v>0</v>
       </c>
     </row>
     <row r="22" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="13">
+      <c r="A22" s="15">
         <v>0</v>
       </c>
     </row>
     <row r="23" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="13">
+      <c r="A23" s="15">
         <v>3</v>
       </c>
     </row>
     <row r="24" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="13">
+      <c r="A24" s="15">
         <v>1</v>
       </c>
     </row>
     <row r="25" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="13">
+      <c r="A25" s="15">
         <v>1</v>
       </c>
     </row>
     <row r="26" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="13">
+      <c r="A26" s="15">
         <v>1</v>
       </c>
     </row>
     <row r="27" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="13">
+      <c r="A27" s="15">
         <v>0</v>
       </c>
     </row>
     <row r="28" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="13">
+      <c r="A28" s="15">
         <v>0</v>
       </c>
     </row>
     <row r="29" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="13">
+      <c r="A29" s="15">
         <v>2</v>
       </c>
     </row>
     <row r="30" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="13">
+      <c r="A30" s="15">
         <v>1</v>
       </c>
     </row>
     <row r="31" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="13">
+      <c r="A31" s="15">
         <v>1</v>
       </c>
     </row>
     <row r="32" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="13">
+      <c r="A32" s="15">
         <v>0</v>
       </c>
     </row>
     <row r="33" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="13">
+      <c r="A33" s="15">
         <v>2</v>
       </c>
     </row>
     <row r="34" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="13">
+      <c r="A34" s="15">
         <v>0</v>
       </c>
     </row>
     <row r="35" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="13">
+      <c r="A35" s="15">
         <v>0</v>
       </c>
     </row>
     <row r="36" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A36" s="13">
+      <c r="A36" s="15">
         <v>1</v>
       </c>
     </row>
     <row r="37" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A37" s="13">
+      <c r="A37" s="15">
         <v>1</v>
       </c>
     </row>
     <row r="38" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A38" s="13">
+      <c r="A38" s="15">
         <v>2</v>
       </c>
     </row>
     <row r="39" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A39" s="13">
+      <c r="A39" s="15">
         <v>2</v>
       </c>
     </row>
     <row r="40" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A40" s="13">
+      <c r="A40" s="15">
         <v>1</v>
       </c>
     </row>
     <row r="41" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A41" s="13">
+      <c r="A41" s="15">
         <v>0</v>
       </c>
     </row>
@@ -1760,7 +1772,7 @@
 </file>
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4F5C6A05-4757-449F-92C5-3840908DD25E}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A1D4F0F4-EC3C-410F-84CD-7E0400989CDB}">
   <dimension ref="A1:D7"/>
   <sheetFormatPr defaultRowHeight="14.3" x14ac:dyDescent="0.25"/>
   <cols>
@@ -1770,55 +1782,55 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="46.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="4" t="s">
         <v>88</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="14" t="s">
+      <c r="D1" s="16" t="s">
         <v>76</v>
       </c>
     </row>
     <row r="2" spans="1:4" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="13" t="s">
+      <c r="A2" s="15" t="s">
         <v>103</v>
       </c>
-      <c r="B2" s="13">
+      <c r="B2" s="15">
         <v>200</v>
       </c>
-      <c r="D2" s="15" t="s">
+      <c r="D2" s="18" t="s">
         <v>106</v>
       </c>
     </row>
     <row r="3" spans="1:4" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="13" t="s">
+      <c r="A3" s="15" t="s">
         <v>104</v>
       </c>
-      <c r="B3" s="13">
+      <c r="B3" s="15">
         <v>0.6</v>
       </c>
-      <c r="D3" s="15"/>
+      <c r="D3" s="17"/>
     </row>
     <row r="4" spans="1:4" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="13" t="s">
+      <c r="A4" s="15" t="s">
         <v>105</v>
       </c>
-      <c r="B4" s="13">
+      <c r="B4" s="15">
         <v>135</v>
       </c>
-      <c r="D4" s="15" t="s">
+      <c r="D4" s="18" t="s">
         <v>107</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D5" s="15"/>
+      <c r="D5" s="17"/>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D6" s="15"/>
+      <c r="D6" s="17"/>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D7" s="15"/>
+      <c r="D7" s="17"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -1830,7 +1842,7 @@
 </file>
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5AF456F1-C8F8-4D4E-8014-33CA30D59399}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A16010E6-9801-407F-982B-0FCC5436B97C}">
   <dimension ref="A1:D7"/>
   <sheetFormatPr defaultRowHeight="14.3" x14ac:dyDescent="0.25"/>
   <cols>
@@ -1839,49 +1851,49 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="46.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="4" t="s">
         <v>88</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="14" t="s">
+      <c r="D1" s="16" t="s">
         <v>76</v>
       </c>
     </row>
     <row r="2" spans="1:4" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="13" t="s">
+      <c r="A2" s="15" t="s">
         <v>108</v>
       </c>
-      <c r="B2" s="13">
+      <c r="B2" s="15">
         <v>100</v>
       </c>
-      <c r="D2" s="15" t="s">
+      <c r="D2" s="18" t="s">
         <v>110</v>
       </c>
     </row>
     <row r="3" spans="1:4" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="13" t="s">
+      <c r="A3" s="15" t="s">
         <v>109</v>
       </c>
-      <c r="B3" s="13">
+      <c r="B3" s="15">
         <v>3</v>
       </c>
-      <c r="D3" s="15"/>
+      <c r="D3" s="17"/>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D4" s="15" t="s">
+      <c r="D4" s="18" t="s">
         <v>111</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D5" s="15"/>
+      <c r="D5" s="17"/>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D6" s="15"/>
+      <c r="D6" s="17"/>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D7" s="15"/>
+      <c r="D7" s="17"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -1893,7 +1905,7 @@
 </file>
 
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D59568EB-F627-493E-BE1B-1B1F6DE6CF06}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E6E1538D-96D4-491C-BB64-4F1305E6B691}">
   <dimension ref="A1:D7"/>
   <sheetFormatPr defaultRowHeight="14.3" x14ac:dyDescent="0.25"/>
   <cols>
@@ -1902,61 +1914,61 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="46.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="4" t="s">
         <v>112</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="4" t="s">
+        <v>113</v>
+      </c>
+      <c r="D1" s="16" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="15" t="s">
+        <v>114</v>
+      </c>
+      <c r="B2" s="15">
+        <v>24</v>
+      </c>
+      <c r="D2" s="18" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="15" t="s">
+        <v>115</v>
+      </c>
+      <c r="B3" s="15">
+        <v>18</v>
+      </c>
+      <c r="D3" s="17"/>
+    </row>
+    <row r="4" spans="1:4" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="15" t="s">
+        <v>116</v>
+      </c>
+      <c r="B4" s="15">
+        <v>12</v>
+      </c>
+      <c r="D4" s="18" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="15" t="s">
         <v>117</v>
       </c>
-      <c r="D1" s="14" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="13" t="s">
-        <v>113</v>
-      </c>
-      <c r="B2" s="13">
-        <v>24</v>
-      </c>
-      <c r="D2" s="15" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="13" t="s">
-        <v>114</v>
-      </c>
-      <c r="B3" s="13">
-        <v>18</v>
-      </c>
-      <c r="D3" s="15"/>
-    </row>
-    <row r="4" spans="1:4" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="13" t="s">
-        <v>115</v>
-      </c>
-      <c r="B4" s="13">
-        <v>12</v>
-      </c>
-      <c r="D4" s="15" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="13" t="s">
-        <v>116</v>
-      </c>
-      <c r="B5" s="13">
+      <c r="B5" s="15">
         <v>6</v>
       </c>
-      <c r="D5" s="15"/>
+      <c r="D5" s="17"/>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D6" s="15"/>
+      <c r="D6" s="17"/>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D7" s="15"/>
+      <c r="D7" s="17"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -1968,7 +1980,7 @@
 </file>
 
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8556A20C-D1B0-4626-B163-CB7F92A83BF3}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A09802A0-45B7-435A-AE00-F026207B7B23}">
   <dimension ref="A1:E7"/>
   <sheetFormatPr defaultRowHeight="14.3" x14ac:dyDescent="0.25"/>
   <cols>
@@ -1977,58 +1989,58 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="46.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="4" t="s">
         <v>120</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="4" t="s">
+        <v>121</v>
+      </c>
+      <c r="C1" s="4" t="s">
+        <v>122</v>
+      </c>
+      <c r="E1" s="16" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="15" t="s">
         <v>123</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="B2" s="15">
+        <v>54</v>
+      </c>
+      <c r="C2" s="15">
+        <v>26</v>
+      </c>
+      <c r="E2" s="18" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="15" t="s">
         <v>124</v>
       </c>
-      <c r="E1" s="14" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="13" t="s">
-        <v>121</v>
-      </c>
-      <c r="B2" s="13">
-        <v>54</v>
-      </c>
-      <c r="C2" s="13">
-        <v>26</v>
-      </c>
-      <c r="E2" s="15" t="s">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="13" t="s">
-        <v>122</v>
-      </c>
-      <c r="B3" s="13">
+      <c r="B3" s="15">
         <v>27</v>
       </c>
-      <c r="C3" s="13">
+      <c r="C3" s="15">
         <v>43</v>
       </c>
-      <c r="E3" s="15"/>
+      <c r="E3" s="17"/>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="E4" s="15" t="s">
+      <c r="E4" s="18" t="s">
         <v>126</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="E5" s="15"/>
+      <c r="E5" s="17"/>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="E6" s="15"/>
+      <c r="E6" s="17"/>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="E7" s="15"/>
+      <c r="E7" s="17"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -2040,7 +2052,7 @@
 </file>
 
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3BFF21B6-C8ED-40CE-BE13-4042EE00BFAF}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B9CBC292-AB2B-438A-8B2D-4C7EA7D6C624}">
   <dimension ref="A1:D7"/>
   <sheetFormatPr defaultRowHeight="14.3" x14ac:dyDescent="0.25"/>
   <cols>
@@ -2050,61 +2062,61 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="46.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="4" t="s">
         <v>88</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="14" t="s">
+      <c r="D1" s="16" t="s">
         <v>76</v>
       </c>
     </row>
     <row r="2" spans="1:4" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="13" t="s">
+      <c r="A2" s="15" t="s">
         <v>95</v>
       </c>
-      <c r="B2" s="13">
+      <c r="B2" s="15">
         <v>4</v>
       </c>
-      <c r="D2" s="15" t="s">
+      <c r="D2" s="18" t="s">
         <v>130</v>
       </c>
     </row>
     <row r="3" spans="1:4" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="13" t="s">
+      <c r="A3" s="15" t="s">
         <v>127</v>
       </c>
-      <c r="B3" s="13">
+      <c r="B3" s="15">
         <v>2</v>
       </c>
-      <c r="D3" s="15"/>
+      <c r="D3" s="17"/>
     </row>
     <row r="4" spans="1:4" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="13" t="s">
+      <c r="A4" s="15" t="s">
         <v>128</v>
       </c>
-      <c r="B4" s="13">
+      <c r="B4" s="15">
         <v>10</v>
       </c>
-      <c r="D4" s="15" t="s">
+      <c r="D4" s="18" t="s">
         <v>131</v>
       </c>
     </row>
     <row r="5" spans="1:4" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="13" t="s">
+      <c r="A5" s="15" t="s">
         <v>129</v>
       </c>
-      <c r="B5" s="13">
+      <c r="B5" s="15">
         <v>4</v>
       </c>
-      <c r="D5" s="15"/>
+      <c r="D5" s="17"/>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D6" s="15"/>
+      <c r="D6" s="17"/>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D7" s="15"/>
+      <c r="D7" s="17"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -2116,7 +2128,7 @@
 </file>
 
 <file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0A0842B4-7EBB-4C5D-A38C-6C26EFB69984}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{742DD14A-1827-43F4-8D10-2943B4E470BA}">
   <dimension ref="A1:D7"/>
   <sheetFormatPr defaultRowHeight="14.3" x14ac:dyDescent="0.25"/>
   <cols>
@@ -2126,67 +2138,67 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="46.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="4" t="s">
         <v>88</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="14" t="s">
+      <c r="D1" s="16" t="s">
         <v>76</v>
       </c>
     </row>
     <row r="2" spans="1:4" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="13" t="s">
+      <c r="A2" s="15" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="13">
+      <c r="B2" s="15">
         <v>1000</v>
       </c>
-      <c r="D2" s="15" t="s">
+      <c r="D2" s="18" t="s">
         <v>134</v>
       </c>
     </row>
     <row r="3" spans="1:4" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="13" t="s">
+      <c r="A3" s="15" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="13">
+      <c r="B3" s="15">
         <v>0.8</v>
       </c>
-      <c r="D3" s="15"/>
+      <c r="D3" s="17"/>
     </row>
     <row r="4" spans="1:4" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="13" t="s">
+      <c r="A4" s="15" t="s">
         <v>5</v>
       </c>
-      <c r="B4" s="13">
+      <c r="B4" s="15">
         <v>0.9</v>
       </c>
-      <c r="D4" s="15" t="s">
+      <c r="D4" s="18" t="s">
         <v>135</v>
       </c>
     </row>
     <row r="5" spans="1:4" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="13" t="s">
+      <c r="A5" s="15" t="s">
         <v>132</v>
       </c>
-      <c r="B5" s="13">
+      <c r="B5" s="15">
         <v>0.05</v>
       </c>
-      <c r="D5" s="15"/>
+      <c r="D5" s="17"/>
     </row>
     <row r="6" spans="1:4" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="13" t="s">
+      <c r="A6" s="15" t="s">
         <v>133</v>
       </c>
-      <c r="B6" s="13">
+      <c r="B6" s="15">
         <v>0.2</v>
       </c>
-      <c r="D6" s="15"/>
+      <c r="D6" s="17"/>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D7" s="15"/>
+      <c r="D7" s="17"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -2198,7 +2210,7 @@
 </file>
 
 <file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C03C4F6C-3E49-4FEE-A0DE-F5BB05C050BE}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{93B02B4F-18CF-4E40-B272-02CD8B78B9BD}">
   <dimension ref="A1:D7"/>
   <sheetFormatPr defaultRowHeight="14.3" x14ac:dyDescent="0.25"/>
   <cols>
@@ -2208,55 +2220,55 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="46.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="4" t="s">
         <v>88</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="14" t="s">
+      <c r="D1" s="16" t="s">
         <v>76</v>
       </c>
     </row>
     <row r="2" spans="1:4" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="13" t="s">
+      <c r="A2" s="15" t="s">
         <v>136</v>
       </c>
-      <c r="B2" s="13">
+      <c r="B2" s="15">
         <v>0.85</v>
       </c>
-      <c r="D2" s="15" t="s">
+      <c r="D2" s="18" t="s">
         <v>139</v>
       </c>
     </row>
     <row r="3" spans="1:4" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="13" t="s">
+      <c r="A3" s="15" t="s">
         <v>137</v>
       </c>
-      <c r="B3" s="13">
+      <c r="B3" s="15">
         <v>0.15</v>
       </c>
-      <c r="D3" s="15"/>
+      <c r="D3" s="17"/>
     </row>
     <row r="4" spans="1:4" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="13" t="s">
+      <c r="A4" s="15" t="s">
         <v>138</v>
       </c>
-      <c r="B4" s="13">
+      <c r="B4" s="15">
         <v>0.8</v>
       </c>
-      <c r="D4" s="15" t="s">
+      <c r="D4" s="18" t="s">
         <v>140</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D5" s="15"/>
+      <c r="D5" s="17"/>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D6" s="15"/>
+      <c r="D6" s="17"/>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D7" s="15"/>
+      <c r="D7" s="17"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -2268,7 +2280,7 @@
 </file>
 
 <file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5B661506-7AC8-4A8B-9DEB-1ADEB1D49C63}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3BBEBF62-EF3B-4F8C-BA7A-8EA32AD8381C}">
   <dimension ref="A1:E7"/>
   <sheetFormatPr defaultRowHeight="14.3" x14ac:dyDescent="0.25"/>
   <cols>
@@ -2277,76 +2289,76 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="46.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="4" t="s">
         <v>141</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="4" t="s">
         <v>142</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C1" s="4" t="s">
         <v>143</v>
       </c>
-      <c r="E1" s="14" t="s">
+      <c r="E1" s="16" t="s">
         <v>76</v>
       </c>
     </row>
     <row r="2" spans="1:5" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="13">
+      <c r="A2" s="15">
         <v>0</v>
       </c>
-      <c r="B2" s="13">
+      <c r="B2" s="15">
         <v>0.1</v>
       </c>
-      <c r="C2" s="13">
+      <c r="C2" s="15">
         <v>3</v>
       </c>
-      <c r="E2" s="15" t="s">
+      <c r="E2" s="18" t="s">
         <v>144</v>
       </c>
     </row>
     <row r="3" spans="1:5" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="13">
+      <c r="A3" s="15">
         <v>1</v>
       </c>
-      <c r="B3" s="13">
+      <c r="B3" s="15">
         <v>0.4</v>
       </c>
-      <c r="C3" s="13">
+      <c r="C3" s="15">
         <v>7</v>
       </c>
-      <c r="E3" s="15"/>
+      <c r="E3" s="17"/>
     </row>
     <row r="4" spans="1:5" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="13">
+      <c r="A4" s="15">
         <v>2</v>
       </c>
-      <c r="B4" s="13">
+      <c r="B4" s="15">
         <v>0.35</v>
       </c>
-      <c r="C4" s="13">
+      <c r="C4" s="15">
         <v>8</v>
       </c>
-      <c r="E4" s="15" t="s">
+      <c r="E4" s="18" t="s">
         <v>145</v>
       </c>
     </row>
     <row r="5" spans="1:5" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="13">
+      <c r="A5" s="15">
         <v>3</v>
       </c>
-      <c r="B5" s="13">
+      <c r="B5" s="15">
         <v>0.15</v>
       </c>
-      <c r="C5" s="13">
+      <c r="C5" s="15">
         <v>2</v>
       </c>
-      <c r="E5" s="15"/>
+      <c r="E5" s="17"/>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="E6" s="15"/>
+      <c r="E6" s="17"/>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="E7" s="15"/>
+      <c r="E7" s="17"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -2358,188 +2370,287 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6F1C5152-8E33-4FA1-B4D1-5320747CA676}">
-  <dimension ref="A1:D20"/>
-  <sheetFormatPr defaultRowHeight="13.6" x14ac:dyDescent="0.25"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4300F14A-94F8-4C1E-9476-0BE1C3844366}">
+  <dimension ref="A1:F22"/>
+  <sheetFormatPr defaultRowHeight="14.3" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="46.625" style="1" customWidth="1"/>
-    <col min="2" max="2" width="14.625" style="1" customWidth="1"/>
-    <col min="3" max="3" width="3.625" style="1" customWidth="1"/>
-    <col min="4" max="4" width="58.625" style="1" customWidth="1"/>
-    <col min="5" max="16384" width="9" style="1"/>
+    <col min="1" max="1" width="46.625" customWidth="1"/>
+    <col min="2" max="2" width="14.625" customWidth="1"/>
+    <col min="3" max="3" width="3.625" customWidth="1"/>
+    <col min="4" max="4" width="58.625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="34" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="2" t="s">
+    <row r="1" spans="1:6" ht="34" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="4" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A2" s="1" t="s">
+      <c r="C1" s="1"/>
+      <c r="D1" s="1"/>
+      <c r="E1" s="1"/>
+      <c r="F1" s="1"/>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="3">
+      <c r="B2" s="5">
         <v>1000</v>
       </c>
-      <c r="D2" s="7" t="s">
+      <c r="C2" s="1"/>
+      <c r="D2" s="9" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A3" s="1" t="s">
+      <c r="E2" s="1"/>
+      <c r="F2" s="1"/>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="4">
+      <c r="B3" s="6">
         <v>0.1</v>
       </c>
-      <c r="D3" s="7" t="s">
+      <c r="C3" s="1"/>
+      <c r="D3" s="9" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A4" s="1" t="s">
+      <c r="E3" s="1"/>
+      <c r="F3" s="1"/>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="B4" s="4">
+      <c r="B4" s="6">
         <v>0.95</v>
       </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A5" s="1" t="s">
+      <c r="C4" s="1"/>
+      <c r="D4" s="1"/>
+      <c r="E4" s="1"/>
+      <c r="F4" s="1"/>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="B5" s="4">
+      <c r="B5" s="6">
         <v>0.9</v>
       </c>
-      <c r="D5" s="7" t="s">
+      <c r="C5" s="1"/>
+      <c r="D5" s="9" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A7" s="1" t="s">
+      <c r="E5" s="1"/>
+      <c r="F5" s="1"/>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A6" s="1"/>
+      <c r="B6" s="1"/>
+      <c r="C6" s="1"/>
+      <c r="D6" s="1"/>
+      <c r="E6" s="1"/>
+      <c r="F6" s="1"/>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A7" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="B7" s="5">
+      <c r="B7" s="7">
         <f>B2*B3</f>
         <v>100</v>
       </c>
-      <c r="D7" s="7" t="s">
+      <c r="C7" s="1"/>
+      <c r="D7" s="9" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A8" s="1" t="s">
+      <c r="E7" s="1"/>
+      <c r="F7" s="1"/>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A8" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="B8" s="5">
+      <c r="B8" s="7">
         <f>B2-B7</f>
         <v>900</v>
       </c>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A9" s="1" t="s">
+      <c r="C8" s="1"/>
+      <c r="D8" s="1"/>
+      <c r="E8" s="1"/>
+      <c r="F8" s="1"/>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A9" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="B9" s="5">
+      <c r="B9" s="7">
         <f>B7*B4</f>
         <v>95</v>
       </c>
-      <c r="D9" s="7" t="s">
+      <c r="C9" s="1"/>
+      <c r="D9" s="9" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A10" s="1" t="s">
+      <c r="E9" s="1"/>
+      <c r="F9" s="1"/>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A10" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="B10" s="5">
+      <c r="B10" s="7">
         <f>B7-B9</f>
         <v>5</v>
       </c>
-      <c r="D10" s="7" t="s">
+      <c r="C10" s="1"/>
+      <c r="D10" s="9" t="s">
         <v>23</v>
       </c>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A11" s="1" t="s">
+      <c r="E10" s="1"/>
+      <c r="F10" s="1"/>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A11" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="B11" s="5">
+      <c r="B11" s="7">
         <f>B8*(1-B5)</f>
         <v>89.999999999999986</v>
       </c>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A12" s="1" t="s">
+      <c r="C11" s="1"/>
+      <c r="D11" s="1"/>
+      <c r="E11" s="1"/>
+      <c r="F11" s="1"/>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A12" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="B12" s="5">
+      <c r="B12" s="7">
         <f>B8-B11</f>
         <v>810</v>
       </c>
-    </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A13" s="1" t="s">
+      <c r="C12" s="1"/>
+      <c r="D12" s="1"/>
+      <c r="E12" s="1"/>
+      <c r="F12" s="1"/>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A13" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="B13" s="5">
+      <c r="B13" s="7">
         <f>B9+B11</f>
         <v>185</v>
       </c>
-    </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A14" s="1" t="s">
+      <c r="C13" s="1"/>
+      <c r="D13" s="1"/>
+      <c r="E13" s="1"/>
+      <c r="F13" s="1"/>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A14" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="B14" s="5">
+      <c r="B14" s="7">
         <f>B10+B12</f>
         <v>815</v>
       </c>
-    </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A16" s="1" t="s">
+      <c r="C14" s="1"/>
+      <c r="D14" s="1"/>
+      <c r="E14" s="1"/>
+      <c r="F14" s="1"/>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A15" s="1"/>
+      <c r="B15" s="1"/>
+      <c r="C15" s="1"/>
+      <c r="D15" s="1"/>
+      <c r="E15" s="1"/>
+      <c r="F15" s="1"/>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A16" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="B16" s="6">
+      <c r="B16" s="8">
         <f>B9/B13</f>
         <v>0.51351351351351349</v>
       </c>
-      <c r="D16" s="7" t="s">
+      <c r="C16" s="1"/>
+      <c r="D16" s="9" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A17" s="1" t="s">
+      <c r="E16" s="1"/>
+      <c r="F16" s="1"/>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A17" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="B17" s="6">
+      <c r="B17" s="8">
         <f>B12/B14</f>
         <v>0.99386503067484666</v>
       </c>
-    </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A19" s="1" t="s">
+      <c r="C17" s="1"/>
+      <c r="D17" s="1"/>
+      <c r="E17" s="1"/>
+      <c r="F17" s="1"/>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A18" s="1"/>
+      <c r="B18" s="1"/>
+      <c r="C18" s="1"/>
+      <c r="D18" s="1"/>
+      <c r="E18" s="1"/>
+      <c r="F18" s="1"/>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A19" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="B19" s="6">
+      <c r="B19" s="8">
         <f>B3*B4+(1-B3)*(1-B5)</f>
         <v>0.185</v>
       </c>
-      <c r="D19" s="7" t="s">
+      <c r="C19" s="1"/>
+      <c r="D19" s="9" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A20" s="1" t="s">
+      <c r="E19" s="1"/>
+      <c r="F19" s="1"/>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A20" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="B20" s="6">
+      <c r="B20" s="8">
         <f>B3*B4/B19</f>
         <v>0.51351351351351349</v>
       </c>
+      <c r="C20" s="1"/>
+      <c r="D20" s="1"/>
+      <c r="E20" s="1"/>
+      <c r="F20" s="1"/>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A21" s="1"/>
+      <c r="B21" s="1"/>
+      <c r="C21" s="1"/>
+      <c r="D21" s="1"/>
+      <c r="E21" s="1"/>
+      <c r="F21" s="1"/>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A22" s="1"/>
+      <c r="B22" s="1"/>
+      <c r="C22" s="1"/>
+      <c r="D22" s="1"/>
+      <c r="E22" s="1"/>
+      <c r="F22" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
@@ -2547,7 +2658,7 @@
 </file>
 
 <file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{680733A0-B8E2-4837-8E18-D82DB08D0A7C}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{73E5AB1F-EB8D-4C08-913B-AD1A98B8E68F}">
   <dimension ref="A1:D7"/>
   <sheetFormatPr defaultRowHeight="14.3" x14ac:dyDescent="0.25"/>
   <cols>
@@ -2557,55 +2668,55 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="46.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="4" t="s">
         <v>88</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="14" t="s">
+      <c r="D1" s="16" t="s">
         <v>76</v>
       </c>
     </row>
     <row r="2" spans="1:4" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="13" t="s">
+      <c r="A2" s="15" t="s">
         <v>146</v>
       </c>
-      <c r="B2" s="13">
+      <c r="B2" s="15">
         <v>4</v>
       </c>
-      <c r="D2" s="15" t="s">
+      <c r="D2" s="18" t="s">
         <v>148</v>
       </c>
     </row>
     <row r="3" spans="1:4" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="13" t="s">
+      <c r="A3" s="15" t="s">
         <v>96</v>
       </c>
-      <c r="B3" s="13">
+      <c r="B3" s="15">
         <v>0.5</v>
       </c>
-      <c r="D3" s="15"/>
+      <c r="D3" s="17"/>
     </row>
     <row r="4" spans="1:4" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="13" t="s">
+      <c r="A4" s="15" t="s">
         <v>147</v>
       </c>
-      <c r="B4" s="13">
+      <c r="B4" s="15">
         <v>3</v>
       </c>
-      <c r="D4" s="15" t="s">
+      <c r="D4" s="18" t="s">
         <v>131</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D5" s="15"/>
+      <c r="D5" s="17"/>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D6" s="15"/>
+      <c r="D6" s="17"/>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D7" s="15"/>
+      <c r="D7" s="17"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -2617,7 +2728,7 @@
 </file>
 
 <file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9C217393-349B-4318-95E4-D25117FB8944}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C97D83DC-8C83-4463-8EE0-4F9AE08333E6}">
   <dimension ref="A1:D7"/>
   <sheetFormatPr defaultRowHeight="14.3" x14ac:dyDescent="0.25"/>
   <cols>
@@ -2627,61 +2738,61 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="46.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="4" t="s">
         <v>88</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="14" t="s">
+      <c r="D1" s="16" t="s">
         <v>76</v>
       </c>
     </row>
     <row r="2" spans="1:4" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="13" t="s">
+      <c r="A2" s="15" t="s">
         <v>146</v>
       </c>
-      <c r="B2" s="13">
+      <c r="B2" s="15">
         <v>15</v>
       </c>
-      <c r="D2" s="15" t="s">
+      <c r="D2" s="18" t="s">
         <v>149</v>
       </c>
     </row>
     <row r="3" spans="1:4" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="13" t="s">
+      <c r="A3" s="15" t="s">
         <v>95</v>
       </c>
-      <c r="B3" s="13">
+      <c r="B3" s="15">
         <v>5</v>
       </c>
-      <c r="D3" s="15"/>
+      <c r="D3" s="17"/>
     </row>
     <row r="4" spans="1:4" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="13" t="s">
+      <c r="A4" s="15" t="s">
         <v>46</v>
       </c>
-      <c r="B4" s="13">
+      <c r="B4" s="15">
         <v>3</v>
       </c>
-      <c r="D4" s="15" t="s">
+      <c r="D4" s="18" t="s">
         <v>131</v>
       </c>
     </row>
     <row r="5" spans="1:4" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="13" t="s">
+      <c r="A5" s="15" t="s">
         <v>47</v>
       </c>
-      <c r="B5" s="13">
+      <c r="B5" s="15">
         <v>7</v>
       </c>
-      <c r="D5" s="15"/>
+      <c r="D5" s="17"/>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D6" s="15"/>
+      <c r="D6" s="17"/>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D7" s="15"/>
+      <c r="D7" s="17"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -2693,7 +2804,7 @@
 </file>
 
 <file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3C6BC7E1-19C0-426F-AE4D-9B922116EEF4}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B1725C09-B1DF-4BB8-B36A-4C11DFB0EBB6}">
   <dimension ref="A1:D7"/>
   <sheetFormatPr defaultRowHeight="14.3" x14ac:dyDescent="0.25"/>
   <cols>
@@ -2703,55 +2814,55 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="46.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="4" t="s">
         <v>88</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="14" t="s">
+      <c r="D1" s="16" t="s">
         <v>76</v>
       </c>
     </row>
     <row r="2" spans="1:4" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="13" t="s">
+      <c r="A2" s="15" t="s">
         <v>146</v>
       </c>
-      <c r="B2" s="13">
+      <c r="B2" s="15">
         <v>100</v>
       </c>
-      <c r="D2" s="15" t="s">
+      <c r="D2" s="18" t="s">
         <v>150</v>
       </c>
     </row>
     <row r="3" spans="1:4" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="13" t="s">
+      <c r="A3" s="15" t="s">
         <v>96</v>
       </c>
-      <c r="B3" s="13">
+      <c r="B3" s="15">
         <v>0.5</v>
       </c>
-      <c r="D3" s="15"/>
+      <c r="D3" s="17"/>
     </row>
     <row r="4" spans="1:4" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="13" t="s">
+      <c r="A4" s="15" t="s">
         <v>105</v>
       </c>
-      <c r="B4" s="13">
+      <c r="B4" s="15">
         <v>65</v>
       </c>
-      <c r="D4" s="15" t="s">
+      <c r="D4" s="18" t="s">
         <v>151</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D5" s="15"/>
+      <c r="D5" s="17"/>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D6" s="15"/>
+      <c r="D6" s="17"/>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D7" s="15"/>
+      <c r="D7" s="17"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -2763,228 +2874,319 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C8CE2F10-6F44-4F90-B94B-6A0ADC90AA22}">
-  <dimension ref="A1:F19"/>
-  <sheetFormatPr defaultRowHeight="13.6" x14ac:dyDescent="0.25"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5A915078-AB32-4DB1-BDD0-8A42E11D13A4}">
+  <dimension ref="A1:F22"/>
+  <sheetFormatPr defaultRowHeight="14.3" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="34.625" style="1" customWidth="1"/>
-    <col min="2" max="4" width="14.625" style="1" customWidth="1"/>
-    <col min="5" max="5" width="3.625" style="1" customWidth="1"/>
-    <col min="6" max="6" width="52.625" style="1" customWidth="1"/>
-    <col min="7" max="16384" width="9" style="1"/>
+    <col min="1" max="1" width="34.625" customWidth="1"/>
+    <col min="2" max="4" width="14.625" customWidth="1"/>
+    <col min="5" max="5" width="3.625" customWidth="1"/>
+    <col min="6" max="6" width="52.625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="34" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="4" t="s">
         <v>1</v>
       </c>
+      <c r="C1" s="1"/>
+      <c r="D1" s="1"/>
+      <c r="E1" s="1"/>
+      <c r="F1" s="1"/>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A2" s="1" t="s">
+      <c r="A2" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="B2" s="8">
+      <c r="B2" s="10">
         <v>5</v>
       </c>
-      <c r="F2" s="7" t="s">
+      <c r="C2" s="1"/>
+      <c r="D2" s="1"/>
+      <c r="E2" s="1"/>
+      <c r="F2" s="9" t="s">
         <v>39</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A3" s="1" t="s">
+      <c r="A3" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="B3" s="4">
+      <c r="B3" s="6">
         <v>0.25</v>
       </c>
-      <c r="F3" s="7" t="s">
+      <c r="C3" s="1"/>
+      <c r="D3" s="1"/>
+      <c r="E3" s="1"/>
+      <c r="F3" s="9" t="s">
         <v>40</v>
       </c>
     </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4" s="1"/>
+      <c r="B4" s="1"/>
+      <c r="C4" s="1"/>
+      <c r="D4" s="1"/>
+      <c r="E4" s="1"/>
+      <c r="F4" s="1"/>
+    </row>
     <row r="5" spans="1:6" ht="34" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="2" t="s">
+      <c r="A5" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="B5" s="2" t="s">
+      <c r="B5" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="C5" s="2" t="s">
+      <c r="C5" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="D5" s="2" t="s">
+      <c r="D5" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="F5" s="7" t="s">
+      <c r="E5" s="1"/>
+      <c r="F5" s="9" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A6" s="8">
+      <c r="A6" s="10">
         <v>0</v>
       </c>
-      <c r="B6" s="9">
+      <c r="B6" s="11">
         <f>_xlfn.BINOM.DIST(A6,$B$2,$B$3,FALSE)</f>
         <v>0.23730468750000006</v>
       </c>
-      <c r="C6" s="9">
+      <c r="C6" s="11">
         <f>_xlfn.BINOM.DIST(A6,$B$2,$B$3,TRUE)</f>
         <v>0.23730468750000006</v>
       </c>
-      <c r="D6" s="9">
+      <c r="D6" s="11">
         <f>1-C6+B6</f>
         <v>1</v>
       </c>
+      <c r="E6" s="1"/>
+      <c r="F6" s="1"/>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A7" s="8">
+      <c r="A7" s="10">
         <v>1</v>
       </c>
-      <c r="B7" s="9">
+      <c r="B7" s="11">
         <f>_xlfn.BINOM.DIST(A7,$B$2,$B$3,FALSE)</f>
         <v>0.3955078125</v>
       </c>
-      <c r="C7" s="9">
+      <c r="C7" s="11">
         <f>_xlfn.BINOM.DIST(A7,$B$2,$B$3,TRUE)</f>
         <v>0.6328125</v>
       </c>
-      <c r="D7" s="9">
+      <c r="D7" s="11">
         <f>1-C7+B7</f>
         <v>0.7626953125</v>
       </c>
-      <c r="F7" s="7" t="s">
+      <c r="E7" s="1"/>
+      <c r="F7" s="9" t="s">
         <v>41</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A8" s="8">
+      <c r="A8" s="10">
         <v>2</v>
       </c>
-      <c r="B8" s="9">
+      <c r="B8" s="11">
         <f>_xlfn.BINOM.DIST(A8,$B$2,$B$3,FALSE)</f>
         <v>0.26367187499999994</v>
       </c>
-      <c r="C8" s="9">
+      <c r="C8" s="11">
         <f>_xlfn.BINOM.DIST(A8,$B$2,$B$3,TRUE)</f>
         <v>0.896484375</v>
       </c>
-      <c r="D8" s="9">
+      <c r="D8" s="11">
         <f>1-C8+B8</f>
         <v>0.36718749999999994</v>
       </c>
+      <c r="E8" s="1"/>
+      <c r="F8" s="1"/>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A9" s="8">
+      <c r="A9" s="10">
         <v>3</v>
       </c>
-      <c r="B9" s="9">
+      <c r="B9" s="11">
         <f>_xlfn.BINOM.DIST(A9,$B$2,$B$3,FALSE)</f>
         <v>8.7890625000000042E-2</v>
       </c>
-      <c r="C9" s="9">
+      <c r="C9" s="11">
         <f>_xlfn.BINOM.DIST(A9,$B$2,$B$3,TRUE)</f>
         <v>0.984375</v>
       </c>
-      <c r="D9" s="9">
+      <c r="D9" s="11">
         <f>1-C9+B9</f>
         <v>0.10351562500000004</v>
       </c>
+      <c r="E9" s="1"/>
+      <c r="F9" s="1"/>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A10" s="8">
+      <c r="A10" s="10">
         <v>4</v>
       </c>
-      <c r="B10" s="9">
+      <c r="B10" s="11">
         <f>_xlfn.BINOM.DIST(A10,$B$2,$B$3,FALSE)</f>
         <v>1.4648437500000005E-2</v>
       </c>
-      <c r="C10" s="9">
+      <c r="C10" s="11">
         <f>_xlfn.BINOM.DIST(A10,$B$2,$B$3,TRUE)</f>
         <v>0.9990234375</v>
       </c>
-      <c r="D10" s="9">
+      <c r="D10" s="11">
         <f>1-C10+B10</f>
         <v>1.5625000000000007E-2</v>
       </c>
+      <c r="E10" s="1"/>
+      <c r="F10" s="1"/>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A11" s="8">
+      <c r="A11" s="10">
         <v>5</v>
       </c>
-      <c r="B11" s="9">
+      <c r="B11" s="11">
         <f>_xlfn.BINOM.DIST(A11,$B$2,$B$3,FALSE)</f>
         <v>9.765625E-4</v>
       </c>
-      <c r="C11" s="9">
+      <c r="C11" s="11">
         <f>_xlfn.BINOM.DIST(A11,$B$2,$B$3,TRUE)</f>
         <v>1</v>
       </c>
-      <c r="D11" s="9">
+      <c r="D11" s="11">
         <f>1-C11+B11</f>
         <v>9.765625E-4</v>
       </c>
+      <c r="E11" s="1"/>
+      <c r="F11" s="1"/>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A12" s="1"/>
+      <c r="B12" s="1"/>
+      <c r="C12" s="1"/>
+      <c r="D12" s="1"/>
+      <c r="E12" s="1"/>
+      <c r="F12" s="1"/>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A13" s="1" t="s">
+      <c r="A13" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="B13" s="9">
+      <c r="B13" s="11">
         <f>SUM(B6:B11)</f>
         <v>1</v>
       </c>
-      <c r="F13" s="7" t="s">
+      <c r="C13" s="1"/>
+      <c r="D13" s="1"/>
+      <c r="E13" s="1"/>
+      <c r="F13" s="9" t="s">
         <v>42</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A14" s="1" t="s">
+      <c r="A14" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="B14" s="10">
+      <c r="B14" s="12">
         <f>B2*B3</f>
         <v>1.25</v>
       </c>
+      <c r="C14" s="1"/>
+      <c r="D14" s="1"/>
+      <c r="E14" s="1"/>
+      <c r="F14" s="1"/>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A15" s="1" t="s">
+      <c r="A15" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="B15" s="6">
+      <c r="B15" s="8">
         <f>SQRT(B2*B3*(1-B3))</f>
         <v>0.96824583655185426</v>
       </c>
+      <c r="C15" s="1"/>
+      <c r="D15" s="1"/>
+      <c r="E15" s="1"/>
+      <c r="F15" s="1"/>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A16" s="1"/>
+      <c r="B16" s="1"/>
+      <c r="C16" s="1"/>
+      <c r="D16" s="1"/>
+      <c r="E16" s="1"/>
+      <c r="F16" s="1"/>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A17" s="1" t="s">
+      <c r="A17" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="B17" s="11">
+      <c r="B17" s="13">
         <f>FACT(5)</f>
         <v>120</v>
       </c>
+      <c r="C17" s="1"/>
+      <c r="D17" s="1"/>
+      <c r="E17" s="1"/>
+      <c r="F17" s="1"/>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A18" s="1" t="s">
+      <c r="A18" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="B18" s="11">
+      <c r="B18" s="13">
         <f>COMBIN(5,2)</f>
         <v>10</v>
       </c>
+      <c r="C18" s="1"/>
+      <c r="D18" s="1"/>
+      <c r="E18" s="1"/>
+      <c r="F18" s="1"/>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A19" s="1" t="s">
+      <c r="A19" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="B19" s="9">
+      <c r="B19" s="11">
         <f>B18*B3^2*(1-B3)^3</f>
         <v>0.263671875</v>
       </c>
-      <c r="F19" s="7" t="s">
+      <c r="C19" s="1"/>
+      <c r="D19" s="1"/>
+      <c r="E19" s="1"/>
+      <c r="F19" s="9" t="s">
         <v>43</v>
       </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A20" s="1"/>
+      <c r="B20" s="1"/>
+      <c r="C20" s="1"/>
+      <c r="D20" s="1"/>
+      <c r="E20" s="1"/>
+      <c r="F20" s="1"/>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A21" s="1"/>
+      <c r="B21" s="1"/>
+      <c r="C21" s="1"/>
+      <c r="D21" s="1"/>
+      <c r="E21" s="1"/>
+      <c r="F21" s="1"/>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A22" s="1"/>
+      <c r="B22" s="1"/>
+      <c r="C22" s="1"/>
+      <c r="D22" s="1"/>
+      <c r="E22" s="1"/>
+      <c r="F22" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
@@ -2992,302 +3194,362 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FD0F58EE-471F-41E9-855D-C57FBEE5A0AB}">
-  <dimension ref="A1:E22"/>
-  <sheetFormatPr defaultRowHeight="13.6" x14ac:dyDescent="0.25"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A08F7A72-0170-499C-96C4-717C22BEB5DA}">
+  <dimension ref="A1:F22"/>
+  <sheetFormatPr defaultRowHeight="14.3" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="46.625" style="1" customWidth="1"/>
-    <col min="2" max="2" width="14.625" style="1" customWidth="1"/>
-    <col min="3" max="3" width="3.625" style="1" customWidth="1"/>
-    <col min="4" max="4" width="10.625" style="1" customWidth="1"/>
-    <col min="5" max="5" width="14.625" style="1" customWidth="1"/>
-    <col min="6" max="16384" width="9" style="1"/>
+    <col min="1" max="1" width="46.625" customWidth="1"/>
+    <col min="2" max="2" width="14.625" customWidth="1"/>
+    <col min="3" max="3" width="3.625" customWidth="1"/>
+    <col min="4" max="4" width="10.625" customWidth="1"/>
+    <col min="5" max="5" width="14.625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="34" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="2" t="s">
+    <row r="1" spans="1:6" ht="34" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="4" t="s">
         <v>44</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="C1" s="1"/>
+      <c r="D1" s="4" t="s">
         <v>45</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="E1" s="4" t="s">
         <v>30</v>
       </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A2" s="1" t="s">
+      <c r="F1" s="1"/>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="B2" s="8">
+      <c r="B2" s="10">
         <v>20</v>
       </c>
-      <c r="D2" s="8">
+      <c r="C2" s="1"/>
+      <c r="D2" s="10">
         <v>0</v>
       </c>
-      <c r="E2" s="9">
+      <c r="E2" s="11">
         <f>_xlfn.BINOM.DIST(D2,$B$2,$B$3,FALSE)</f>
         <v>3.1712119389339963E-3</v>
       </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A3" s="1" t="s">
+      <c r="F2" s="1"/>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="B3" s="4">
+      <c r="B3" s="6">
         <v>0.25</v>
       </c>
-      <c r="D3" s="8">
+      <c r="C3" s="1"/>
+      <c r="D3" s="10">
         <v>1</v>
       </c>
-      <c r="E3" s="9">
+      <c r="E3" s="11">
         <f>_xlfn.BINOM.DIST(D3,$B$2,$B$3,FALSE)</f>
         <v>2.1141412926226615E-2</v>
       </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A4" s="1" t="s">
+      <c r="F3" s="1"/>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="B4" s="8">
+      <c r="B4" s="10">
         <v>5</v>
       </c>
-      <c r="D4" s="8">
+      <c r="C4" s="1"/>
+      <c r="D4" s="10">
         <v>2</v>
       </c>
-      <c r="E4" s="9">
+      <c r="E4" s="11">
         <f>_xlfn.BINOM.DIST(D4,$B$2,$B$3,FALSE)</f>
         <v>6.6947807599717662E-2</v>
       </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A5" s="1" t="s">
+      <c r="F4" s="1"/>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="B5" s="8">
+      <c r="B5" s="10">
         <v>10</v>
       </c>
-      <c r="D5" s="8">
+      <c r="C5" s="1"/>
+      <c r="D5" s="10">
         <v>3</v>
       </c>
-      <c r="E5" s="9">
+      <c r="E5" s="11">
         <f>_xlfn.BINOM.DIST(D5,$B$2,$B$3,FALSE)</f>
         <v>0.13389561519943524</v>
       </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="D6" s="8">
+      <c r="F5" s="1"/>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A6" s="1"/>
+      <c r="B6" s="1"/>
+      <c r="C6" s="1"/>
+      <c r="D6" s="10">
         <v>4</v>
       </c>
-      <c r="E6" s="9">
+      <c r="E6" s="11">
         <f>_xlfn.BINOM.DIST(D6,$B$2,$B$3,FALSE)</f>
         <v>0.18968545486586663</v>
       </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A7" s="1" t="s">
+      <c r="F6" s="1"/>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A7" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="B7" s="9">
+      <c r="B7" s="11">
         <f>_xlfn.BINOM.DIST(B4,B2,B3,FALSE)</f>
         <v>0.20233115185692441</v>
       </c>
-      <c r="D7" s="8">
+      <c r="C7" s="1"/>
+      <c r="D7" s="10">
         <v>5</v>
       </c>
-      <c r="E7" s="9">
+      <c r="E7" s="11">
         <f>_xlfn.BINOM.DIST(D7,$B$2,$B$3,FALSE)</f>
         <v>0.20233115185692441</v>
       </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A8" s="1" t="s">
+      <c r="F7" s="1"/>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A8" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="B8" s="9">
+      <c r="B8" s="11">
         <f>_xlfn.BINOM.DIST(B4,B2,B3,TRUE)</f>
         <v>0.61717265438710467</v>
       </c>
-      <c r="D8" s="8">
+      <c r="C8" s="1"/>
+      <c r="D8" s="10">
         <v>6</v>
       </c>
-      <c r="E8" s="9">
+      <c r="E8" s="11">
         <f>_xlfn.BINOM.DIST(D8,$B$2,$B$3,FALSE)</f>
         <v>0.1686092932141037</v>
       </c>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A9" s="1" t="s">
+      <c r="F8" s="1"/>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A9" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="B9" s="9">
+      <c r="B9" s="11">
         <f>1-_xlfn.BINOM.DIST(B5-1,B2,B3,TRUE)</f>
         <v>1.3864416943761171E-2</v>
       </c>
-      <c r="D9" s="8">
+      <c r="C9" s="1"/>
+      <c r="D9" s="10">
         <v>7</v>
       </c>
-      <c r="E9" s="9">
+      <c r="E9" s="11">
         <f>_xlfn.BINOM.DIST(D9,$B$2,$B$3,FALSE)</f>
         <v>0.11240619547606913</v>
       </c>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A10" s="1" t="s">
+      <c r="F9" s="1"/>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A10" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="B10" s="9">
+      <c r="B10" s="11">
         <f>_xlfn.BINOM.DIST.RANGE(B2,B3,B5,B2)</f>
         <v>1.3864416943761178E-2</v>
       </c>
-      <c r="D10" s="8">
+      <c r="C10" s="1"/>
+      <c r="D10" s="10">
         <v>8</v>
       </c>
-      <c r="E10" s="9">
+      <c r="E10" s="11">
         <f>_xlfn.BINOM.DIST(D10,$B$2,$B$3,FALSE)</f>
         <v>6.0886689216204062E-2</v>
       </c>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A11" s="1" t="s">
+      <c r="F10" s="1"/>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A11" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="B11" s="10">
+      <c r="B11" s="12">
         <f>B2*B3</f>
         <v>5</v>
       </c>
-      <c r="D11" s="8">
+      <c r="C11" s="1"/>
+      <c r="D11" s="10">
         <v>9</v>
       </c>
-      <c r="E11" s="9">
+      <c r="E11" s="11">
         <f>_xlfn.BINOM.DIST(D11,$B$2,$B$3,FALSE)</f>
         <v>2.7060750762757369E-2</v>
       </c>
-    </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A12" s="1" t="s">
+      <c r="F11" s="1"/>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A12" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="B12" s="6">
+      <c r="B12" s="8">
         <f>SQRT(B2*B3*(1-B3))</f>
         <v>1.9364916731037085</v>
       </c>
-      <c r="D12" s="8">
+      <c r="C12" s="1"/>
+      <c r="D12" s="10">
         <v>10</v>
       </c>
-      <c r="E12" s="9">
+      <c r="E12" s="11">
         <f>_xlfn.BINOM.DIST(D12,$B$2,$B$3,FALSE)</f>
         <v>9.9222752796777041E-3</v>
       </c>
-    </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A13" s="1" t="s">
+      <c r="F12" s="1"/>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A13" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="B13" s="11">
+      <c r="B13" s="13">
         <f>_xlfn.BINOM.INV(B2,B3,0.95)</f>
         <v>8</v>
       </c>
-      <c r="D13" s="8">
+      <c r="C13" s="1"/>
+      <c r="D13" s="10">
         <v>11</v>
       </c>
-      <c r="E13" s="9">
+      <c r="E13" s="11">
         <f>_xlfn.BINOM.DIST(D13,$B$2,$B$3,FALSE)</f>
         <v>3.0067500847508173E-3</v>
       </c>
-    </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="D14" s="8">
+      <c r="F13" s="1"/>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A14" s="1"/>
+      <c r="B14" s="1"/>
+      <c r="C14" s="1"/>
+      <c r="D14" s="10">
         <v>12</v>
       </c>
-      <c r="E14" s="9">
+      <c r="E14" s="11">
         <f>_xlfn.BINOM.DIST(D14,$B$2,$B$3,FALSE)</f>
         <v>7.5168752118770586E-4</v>
       </c>
-    </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="D15" s="8">
+      <c r="F14" s="1"/>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A15" s="1"/>
+      <c r="B15" s="1"/>
+      <c r="C15" s="1"/>
+      <c r="D15" s="10">
         <v>13</v>
       </c>
-      <c r="E15" s="9">
+      <c r="E15" s="11">
         <f>_xlfn.BINOM.DIST(D15,$B$2,$B$3,FALSE)</f>
         <v>1.541923120385034E-4</v>
       </c>
-    </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A16" s="7" t="s">
+      <c r="F15" s="1"/>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A16" s="9" t="s">
         <v>20</v>
       </c>
-      <c r="D16" s="8">
+      <c r="B16" s="1"/>
+      <c r="C16" s="1"/>
+      <c r="D16" s="10">
         <v>14</v>
       </c>
-      <c r="E16" s="9">
+      <c r="E16" s="11">
         <f>_xlfn.BINOM.DIST(D16,$B$2,$B$3,FALSE)</f>
         <v>2.5698718673083962E-5</v>
       </c>
-    </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A17" s="7" t="s">
+      <c r="F16" s="1"/>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A17" s="9" t="s">
         <v>53</v>
       </c>
-      <c r="D17" s="8">
+      <c r="B17" s="1"/>
+      <c r="C17" s="1"/>
+      <c r="D17" s="10">
         <v>15</v>
       </c>
-      <c r="E17" s="9">
+      <c r="E17" s="11">
         <f>_xlfn.BINOM.DIST(D17,$B$2,$B$3,FALSE)</f>
         <v>3.42649582307786E-6</v>
       </c>
-    </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="D18" s="8">
+      <c r="F17" s="1"/>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A18" s="1"/>
+      <c r="B18" s="1"/>
+      <c r="C18" s="1"/>
+      <c r="D18" s="10">
         <v>16</v>
       </c>
-      <c r="E18" s="9">
+      <c r="E18" s="11">
         <f>_xlfn.BINOM.DIST(D18,$B$2,$B$3,FALSE)</f>
         <v>3.5692664823727645E-7</v>
       </c>
-    </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A19" s="7" t="s">
+      <c r="F18" s="1"/>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A19" s="9" t="s">
         <v>54</v>
       </c>
-      <c r="D19" s="8">
+      <c r="B19" s="1"/>
+      <c r="C19" s="1"/>
+      <c r="D19" s="10">
         <v>17</v>
       </c>
-      <c r="E19" s="9">
+      <c r="E19" s="11">
         <f>_xlfn.BINOM.DIST(D19,$B$2,$B$3,FALSE)</f>
         <v>2.7994246920570738E-8</v>
       </c>
-    </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="D20" s="8">
+      <c r="F19" s="1"/>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A20" s="1"/>
+      <c r="B20" s="1"/>
+      <c r="C20" s="1"/>
+      <c r="D20" s="10">
         <v>18</v>
       </c>
-      <c r="E20" s="9">
+      <c r="E20" s="11">
         <f>_xlfn.BINOM.DIST(D20,$B$2,$B$3,FALSE)</f>
         <v>1.5552359400317114E-9</v>
       </c>
-    </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="D21" s="8">
+      <c r="F20" s="1"/>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A21" s="1"/>
+      <c r="B21" s="1"/>
+      <c r="C21" s="1"/>
+      <c r="D21" s="10">
         <v>19</v>
       </c>
-      <c r="E21" s="9">
+      <c r="E21" s="11">
         <f>_xlfn.BINOM.DIST(D21,$B$2,$B$3,FALSE)</f>
         <v>5.4569682106375856E-11</v>
       </c>
-    </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="D22" s="8">
+      <c r="F21" s="1"/>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A22" s="1"/>
+      <c r="B22" s="1"/>
+      <c r="C22" s="1"/>
+      <c r="D22" s="10">
         <v>20</v>
       </c>
-      <c r="E22" s="9">
+      <c r="E22" s="11">
         <f>_xlfn.BINOM.DIST(D22,$B$2,$B$3,FALSE)</f>
         <v>9.0949470177292824E-13</v>
       </c>
+      <c r="F22" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
@@ -3295,156 +3557,269 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E2A11AF3-D2BC-4585-948D-B13F188B4324}">
-  <dimension ref="A1:D16"/>
-  <sheetFormatPr defaultRowHeight="13.6" x14ac:dyDescent="0.25"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6779A5B5-A1C2-4FD5-9F79-6AFE306BB888}">
+  <dimension ref="A1:F22"/>
+  <sheetFormatPr defaultRowHeight="14.3" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="46.625" style="1" customWidth="1"/>
-    <col min="2" max="2" width="14.625" style="1" customWidth="1"/>
-    <col min="3" max="3" width="3.625" style="1" customWidth="1"/>
-    <col min="4" max="4" width="56.625" style="1" customWidth="1"/>
-    <col min="5" max="16384" width="9" style="1"/>
+    <col min="1" max="1" width="46.625" customWidth="1"/>
+    <col min="2" max="2" width="14.625" customWidth="1"/>
+    <col min="3" max="3" width="3.625" customWidth="1"/>
+    <col min="4" max="4" width="56.625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="34" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="2" t="s">
+    <row r="1" spans="1:6" ht="34" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="4" t="s">
         <v>55</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="4" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A2" s="1" t="s">
+      <c r="C1" s="1"/>
+      <c r="D1" s="1"/>
+      <c r="E1" s="1"/>
+      <c r="F1" s="1"/>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="B2" s="8">
+      <c r="B2" s="10">
         <v>200</v>
       </c>
-      <c r="D2" s="7" t="s">
+      <c r="C2" s="1"/>
+      <c r="D2" s="9" t="s">
         <v>66</v>
       </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A3" s="1" t="s">
+      <c r="E2" s="1"/>
+      <c r="F2" s="1"/>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="B3" s="4">
+      <c r="B3" s="6">
         <v>0.6</v>
       </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A4" s="1" t="s">
+      <c r="C3" s="1"/>
+      <c r="D3" s="1"/>
+      <c r="E3" s="1"/>
+      <c r="F3" s="1"/>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="B4" s="8">
+      <c r="B4" s="10">
         <v>135</v>
       </c>
-      <c r="D4" s="7" t="s">
+      <c r="C4" s="1"/>
+      <c r="D4" s="9" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A6" s="1" t="s">
+      <c r="E4" s="1"/>
+      <c r="F4" s="1"/>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5" s="1"/>
+      <c r="B5" s="1"/>
+      <c r="C5" s="1"/>
+      <c r="D5" s="1"/>
+      <c r="E5" s="1"/>
+      <c r="F5" s="1"/>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A6" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="B6" s="10">
+      <c r="B6" s="12">
         <f>B2*B3</f>
         <v>120</v>
       </c>
-      <c r="D6" s="7" t="s">
+      <c r="C6" s="1"/>
+      <c r="D6" s="9" t="s">
         <v>67</v>
       </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A7" s="1" t="s">
+      <c r="E6" s="1"/>
+      <c r="F6" s="1"/>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A7" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="B7" s="10">
+      <c r="B7" s="12">
         <f>B2*(1-B3)</f>
         <v>80</v>
       </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A8" s="1" t="s">
+      <c r="C7" s="1"/>
+      <c r="D7" s="1"/>
+      <c r="E7" s="1"/>
+      <c r="F7" s="1"/>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A8" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="B8" s="6">
+      <c r="B8" s="8">
         <f>SQRT(B2*B3*(1-B3))</f>
         <v>6.9282032302755088</v>
       </c>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A9" s="1" t="s">
+      <c r="C8" s="1"/>
+      <c r="D8" s="1"/>
+      <c r="E8" s="1"/>
+      <c r="F8" s="1"/>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A9" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="B9" s="6">
+      <c r="B9" s="8">
         <f>(B4-B6)/B8</f>
         <v>2.1650635094610968</v>
       </c>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A10" s="1" t="s">
+      <c r="C9" s="1"/>
+      <c r="D9" s="1"/>
+      <c r="E9" s="1"/>
+      <c r="F9" s="1"/>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A10" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="B10" s="9">
+      <c r="B10" s="11">
         <f>1-_xlfn.NORM.S.DIST(B9,TRUE)</f>
         <v>1.51914109882888E-2</v>
       </c>
-      <c r="D10" s="7" t="s">
+      <c r="C10" s="1"/>
+      <c r="D10" s="9" t="s">
         <v>68</v>
       </c>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A11" s="1" t="s">
+      <c r="E10" s="1"/>
+      <c r="F10" s="1"/>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A11" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="B11" s="9">
+      <c r="B11" s="11">
         <f>1-_xlfn.BINOM.DIST(B4-1,B2,B3,TRUE)</f>
         <v>1.7307341051347791E-2</v>
       </c>
-      <c r="D11" s="7" t="s">
+      <c r="C11" s="1"/>
+      <c r="D11" s="9" t="s">
         <v>69</v>
       </c>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A12" s="1" t="s">
+      <c r="E11" s="1"/>
+      <c r="F11" s="1"/>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A12" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="B12" s="9">
+      <c r="B12" s="11">
         <f>1-_xlfn.NORM.DIST(B4-0.5,B6,B8,TRUE)</f>
         <v>1.8179276586395288E-2</v>
       </c>
-    </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A14" s="1" t="s">
+      <c r="C12" s="1"/>
+      <c r="D12" s="1"/>
+      <c r="E12" s="1"/>
+      <c r="F12" s="1"/>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A13" s="1"/>
+      <c r="B13" s="1"/>
+      <c r="C13" s="1"/>
+      <c r="D13" s="1"/>
+      <c r="E13" s="1"/>
+      <c r="F13" s="1"/>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A14" s="2" t="s">
         <v>63</v>
       </c>
-      <c r="B14" s="6">
+      <c r="B14" s="8">
         <f>B4/B2</f>
         <v>0.67500000000000004</v>
       </c>
-    </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A15" s="1" t="s">
+      <c r="C14" s="1"/>
+      <c r="D14" s="1"/>
+      <c r="E14" s="1"/>
+      <c r="F14" s="1"/>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A15" s="2" t="s">
         <v>64</v>
       </c>
-      <c r="B15" s="12">
+      <c r="B15" s="14">
         <f>SQRT(B3*(1-B3)/B2)</f>
         <v>3.4641016151377546E-2</v>
       </c>
-    </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A16" s="1" t="s">
+      <c r="C15" s="1"/>
+      <c r="D15" s="1"/>
+      <c r="E15" s="1"/>
+      <c r="F15" s="1"/>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A16" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="B16" s="6">
+      <c r="B16" s="8">
         <f>(B14-B3)/B15</f>
         <v>2.1650635094610986</v>
       </c>
-      <c r="D16" s="7" t="s">
+      <c r="C16" s="1"/>
+      <c r="D16" s="9" t="s">
         <v>70</v>
       </c>
+      <c r="E16" s="1"/>
+      <c r="F16" s="1"/>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A17" s="1"/>
+      <c r="B17" s="1"/>
+      <c r="C17" s="1"/>
+      <c r="D17" s="1"/>
+      <c r="E17" s="1"/>
+      <c r="F17" s="1"/>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A18" s="1"/>
+      <c r="B18" s="1"/>
+      <c r="C18" s="1"/>
+      <c r="D18" s="1"/>
+      <c r="E18" s="1"/>
+      <c r="F18" s="1"/>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A19" s="1"/>
+      <c r="B19" s="1"/>
+      <c r="C19" s="1"/>
+      <c r="D19" s="1"/>
+      <c r="E19" s="1"/>
+      <c r="F19" s="1"/>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A20" s="1"/>
+      <c r="B20" s="1"/>
+      <c r="C20" s="1"/>
+      <c r="D20" s="1"/>
+      <c r="E20" s="1"/>
+      <c r="F20" s="1"/>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A21" s="1"/>
+      <c r="B21" s="1"/>
+      <c r="C21" s="1"/>
+      <c r="D21" s="1"/>
+      <c r="E21" s="1"/>
+      <c r="F21" s="1"/>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A22" s="1"/>
+      <c r="B22" s="1"/>
+      <c r="C22" s="1"/>
+      <c r="D22" s="1"/>
+      <c r="E22" s="1"/>
+      <c r="F22" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
@@ -3452,7 +3827,7 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D45E2E77-B09C-4530-AC7A-B3B3AF48A2BD}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{257764B6-587A-470C-8FB3-19CE21906CB0}">
   <dimension ref="A1:D7"/>
   <sheetFormatPr defaultRowHeight="14.3" x14ac:dyDescent="0.25"/>
   <cols>
@@ -3461,55 +3836,55 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="46.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="4" t="s">
         <v>71</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="4" t="s">
+        <v>72</v>
+      </c>
+      <c r="D1" s="16" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="15" t="s">
+        <v>73</v>
+      </c>
+      <c r="B2" s="15">
+        <v>40</v>
+      </c>
+      <c r="D2" s="18" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="15" t="s">
+        <v>74</v>
+      </c>
+      <c r="B3" s="15">
+        <v>35</v>
+      </c>
+      <c r="D3" s="17"/>
+    </row>
+    <row r="4" spans="1:4" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="15" t="s">
         <v>75</v>
       </c>
-      <c r="D1" s="14" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="13" t="s">
-        <v>72</v>
-      </c>
-      <c r="B2" s="13">
-        <v>40</v>
-      </c>
-      <c r="D2" s="15" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="13" t="s">
-        <v>73</v>
-      </c>
-      <c r="B3" s="13">
-        <v>35</v>
-      </c>
-      <c r="D3" s="15"/>
-    </row>
-    <row r="4" spans="1:4" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="13" t="s">
-        <v>74</v>
-      </c>
-      <c r="B4" s="13">
+      <c r="B4" s="15">
         <v>25</v>
       </c>
-      <c r="D4" s="15" t="s">
+      <c r="D4" s="18" t="s">
         <v>78</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D5" s="15"/>
+      <c r="D5" s="17"/>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D6" s="15"/>
+      <c r="D6" s="17"/>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D7" s="15"/>
+      <c r="D7" s="17"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -3521,7 +3896,7 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{01DF041B-942F-4EF5-935C-4C293BDAD3FB}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9C8870F7-321C-499A-B39C-67D64A0C3712}">
   <dimension ref="A1:E7"/>
   <sheetFormatPr defaultRowHeight="14.3" x14ac:dyDescent="0.25"/>
   <cols>
@@ -3530,58 +3905,58 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="46.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="4" t="s">
         <v>79</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="4" t="s">
+        <v>80</v>
+      </c>
+      <c r="C1" s="4" t="s">
+        <v>81</v>
+      </c>
+      <c r="E1" s="16" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="15" t="s">
         <v>82</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="B2" s="15">
+        <v>40</v>
+      </c>
+      <c r="C2" s="15">
+        <v>60</v>
+      </c>
+      <c r="E2" s="18" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="15" t="s">
         <v>83</v>
       </c>
-      <c r="E1" s="14" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="13" t="s">
-        <v>80</v>
-      </c>
-      <c r="B2" s="13">
-        <v>40</v>
-      </c>
-      <c r="C2" s="13">
-        <v>60</v>
-      </c>
-      <c r="E2" s="15" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="13" t="s">
-        <v>81</v>
-      </c>
-      <c r="B3" s="13">
+      <c r="B3" s="15">
         <v>30</v>
       </c>
-      <c r="C3" s="13">
+      <c r="C3" s="15">
         <v>70</v>
       </c>
-      <c r="E3" s="15"/>
+      <c r="E3" s="17"/>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="E4" s="15" t="s">
+      <c r="E4" s="18" t="s">
         <v>85</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="E5" s="15"/>
+      <c r="E5" s="17"/>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="E6" s="15"/>
+      <c r="E6" s="17"/>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="E7" s="15"/>
+      <c r="E7" s="17"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -3593,7 +3968,7 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F0A3D9FB-CF10-4923-AD47-75DE0B24E652}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{428B3A6F-D4FE-47FD-9E25-DC0E9B3A7E07}">
   <dimension ref="A1:E7"/>
   <sheetFormatPr defaultRowHeight="14.3" x14ac:dyDescent="0.25"/>
   <cols>
@@ -3602,58 +3977,58 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="46.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="4" t="s">
         <v>79</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="4" t="s">
+        <v>80</v>
+      </c>
+      <c r="C1" s="4" t="s">
+        <v>81</v>
+      </c>
+      <c r="E1" s="16" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="15" t="s">
         <v>82</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="B2" s="15">
+        <v>30</v>
+      </c>
+      <c r="C2" s="15">
+        <v>70</v>
+      </c>
+      <c r="E2" s="18" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="15" t="s">
         <v>83</v>
       </c>
-      <c r="E1" s="14" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="13" t="s">
-        <v>80</v>
-      </c>
-      <c r="B2" s="13">
+      <c r="B3" s="15">
         <v>30</v>
       </c>
-      <c r="C2" s="13">
+      <c r="C3" s="15">
         <v>70</v>
       </c>
-      <c r="E2" s="15" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="13" t="s">
-        <v>81</v>
-      </c>
-      <c r="B3" s="13">
-        <v>30</v>
-      </c>
-      <c r="C3" s="13">
-        <v>70</v>
-      </c>
-      <c r="E3" s="15"/>
+      <c r="E3" s="17"/>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="E4" s="15" t="s">
+      <c r="E4" s="18" t="s">
         <v>87</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="E5" s="15"/>
+      <c r="E5" s="17"/>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="E6" s="15"/>
+      <c r="E6" s="17"/>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="E7" s="15"/>
+      <c r="E7" s="17"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -3665,7 +4040,7 @@
 </file>
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{064BA3AF-430D-45C4-888E-27C7A3FD99CD}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{68B1D094-92C7-421B-8ED5-20F1D2185A2C}">
   <dimension ref="A1:D7"/>
   <sheetFormatPr defaultRowHeight="14.3" x14ac:dyDescent="0.25"/>
   <cols>
@@ -3675,73 +4050,73 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="46.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="4" t="s">
         <v>88</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="14" t="s">
+      <c r="D1" s="16" t="s">
         <v>76</v>
       </c>
     </row>
     <row r="2" spans="1:4" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="13" t="s">
+      <c r="A2" s="15" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="13">
+      <c r="B2" s="15">
         <v>1000</v>
       </c>
-      <c r="D2" s="15" t="s">
+      <c r="D2" s="18" t="s">
         <v>92</v>
       </c>
     </row>
     <row r="3" spans="1:4" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="13" t="s">
+      <c r="A3" s="15" t="s">
         <v>89</v>
       </c>
-      <c r="B3" s="13">
+      <c r="B3" s="15">
         <v>0.1</v>
       </c>
-      <c r="D3" s="15"/>
+      <c r="D3" s="17"/>
     </row>
     <row r="4" spans="1:4" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="13" t="s">
+      <c r="A4" s="15" t="s">
         <v>4</v>
       </c>
-      <c r="B4" s="13">
+      <c r="B4" s="15">
         <v>0.95</v>
       </c>
-      <c r="D4" s="15" t="s">
+      <c r="D4" s="18" t="s">
         <v>93</v>
       </c>
     </row>
     <row r="5" spans="1:4" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="13" t="s">
+      <c r="A5" s="15" t="s">
         <v>5</v>
       </c>
-      <c r="B5" s="13">
+      <c r="B5" s="15">
         <v>0.9</v>
       </c>
-      <c r="D5" s="15"/>
+      <c r="D5" s="17"/>
     </row>
     <row r="6" spans="1:4" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="13" t="s">
+      <c r="A6" s="15" t="s">
         <v>90</v>
       </c>
-      <c r="B6" s="13">
+      <c r="B6" s="15">
         <v>0.01</v>
       </c>
-      <c r="D6" s="15"/>
+      <c r="D6" s="17"/>
     </row>
     <row r="7" spans="1:4" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="13" t="s">
+      <c r="A7" s="15" t="s">
         <v>91</v>
       </c>
-      <c r="B7" s="13">
+      <c r="B7" s="15">
         <v>10000</v>
       </c>
-      <c r="D7" s="15"/>
+      <c r="D7" s="17"/>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>

<commit_message>
Revise chapter 5 probability explanations and workbook controls
</commit_message>
<xml_diff>
--- a/data/kapitola_05.xlsx
+++ b/data/kapitola_05.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="202300"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{E68C876B-4860-4929-9365-53A085875B78}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{A686227C-91E5-4FD3-8D6B-63257186C438}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-109" yWindow="-109" windowWidth="34995" windowHeight="19060" xr2:uid="{DE02CC22-A075-4BAC-A50D-3760BFE17441}"/>
+    <workbookView xWindow="-109" yWindow="-109" windowWidth="34995" windowHeight="19060" xr2:uid="{99AC8C74-C027-4117-BBC3-80F61B39B3A4}"/>
   </bookViews>
   <sheets>
     <sheet name="Prehled" sheetId="1" r:id="rId1"/>
@@ -55,7 +55,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="296" uniqueCount="196">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="293" uniqueCount="196">
   <si>
     <t>Screening</t>
   </si>
@@ -138,93 +138,90 @@
     <t>Binomický model</t>
   </si>
   <si>
+    <t>Počet pokusů n (pevně)</t>
+  </si>
+  <si>
+    <t>Pravděpodobnost úspěchu π</t>
+  </si>
+  <si>
+    <t>Počet úspěchů k</t>
+  </si>
+  <si>
+    <t>P(X = k)</t>
+  </si>
+  <si>
+    <t>P(X ≤ k)</t>
+  </si>
+  <si>
+    <t>P(X ≥ k)</t>
+  </si>
+  <si>
+    <t>Součet pravděpodobností</t>
+  </si>
+  <si>
+    <t>Střední hodnota</t>
+  </si>
+  <si>
+    <t>Směrodatná odchylka</t>
+  </si>
+  <si>
+    <t>Faktoriál 5!</t>
+  </si>
+  <si>
+    <t>Kombinační číslo 5 nad 2</t>
+  </si>
+  <si>
+    <t>Ruční výpočet P(X = 2)</t>
+  </si>
+  <si>
+    <t>Model náhodného a nezávislého tipování.</t>
+  </si>
+  <si>
+    <t>Počet pokusů je pevně 5 (k od 0 do 5).</t>
+  </si>
+  <si>
+    <t>Měnit lze pouze žlutou B3; ostatní buňky jsou uzamčené.</t>
+  </si>
+  <si>
+    <t>Změnou B3 zjistíte vliv pravděpodobnosti úspěchu.</t>
+  </si>
+  <si>
+    <t>Součet musí být 1.</t>
+  </si>
+  <si>
+    <t>B19 se musí shodovat s B8 i po změně B3.</t>
+  </si>
+  <si>
+    <t>Delší test</t>
+  </si>
+  <si>
+    <t>k</t>
+  </si>
+  <si>
+    <t>Hodnota pro právě a nejvýše</t>
+  </si>
+  <si>
+    <t>Hranice pro alespoň</t>
+  </si>
+  <si>
+    <t>Totéž funkcí BINOM.DIST.RANGE</t>
+  </si>
+  <si>
+    <t>Nejmenší k s P(X ≤ k) alespoň 0,95</t>
+  </si>
+  <si>
+    <t>Měnit lze B3:B5; n = 20 je pevné.</t>
+  </si>
+  <si>
+    <t>Sloupce D a E: celé rozdělení pro n = 20.</t>
+  </si>
+  <si>
+    <t>Normální aproximace</t>
+  </si>
+  <si>
     <t>Počet pokusů n</t>
   </si>
   <si>
-    <t>Pravděpodobnost úspěchu π</t>
-  </si>
-  <si>
-    <t>Počet úspěchů k</t>
-  </si>
-  <si>
-    <t>P(X = k)</t>
-  </si>
-  <si>
-    <t>P(X ≤ k)</t>
-  </si>
-  <si>
-    <t>P(X ≥ k)</t>
-  </si>
-  <si>
-    <t>Součet pravděpodobností</t>
-  </si>
-  <si>
-    <t>Střední hodnota</t>
-  </si>
-  <si>
-    <t>Směrodatná odchylka</t>
-  </si>
-  <si>
-    <t>Faktoriál 5!</t>
-  </si>
-  <si>
-    <t>Kombinační číslo 5 nad 2</t>
-  </si>
-  <si>
-    <t>Ruční výpočet P(X = 2)</t>
-  </si>
-  <si>
-    <t>Model náhodného a nezávislého tipování.</t>
-  </si>
-  <si>
-    <t>Tabulka je připravena pro n = 5 (k od 0 do 5).</t>
-  </si>
-  <si>
-    <t>Změnou B3 zjistíte vliv pravděpodobnosti úspěchu.</t>
-  </si>
-  <si>
-    <t>Součet musí být 1.</t>
-  </si>
-  <si>
-    <t>B19 se má shodovat s B8 při n = 5.</t>
-  </si>
-  <si>
-    <t>Delší test</t>
-  </si>
-  <si>
-    <t>k</t>
-  </si>
-  <si>
-    <t>Hodnota pro právě a nejvýše</t>
-  </si>
-  <si>
-    <t>Hranice pro alespoň</t>
-  </si>
-  <si>
-    <t>Právě: P(X = 5)</t>
-  </si>
-  <si>
-    <t>Nejvýše: P(X ≤ 5)</t>
-  </si>
-  <si>
-    <t>Alespoň: P(X ≥ 10)</t>
-  </si>
-  <si>
-    <t>Totéž funkcí BINOM.DIST.RANGE</t>
-  </si>
-  <si>
-    <t>Nejmenší k s P(X ≤ k) alespoň 0,95</t>
-  </si>
-  <si>
-    <t>Sloupce D a E: celé rozdělení pro n = 20.</t>
-  </si>
-  <si>
-    <t>Alespoň 10 = 1 − nejvýše 9, proto B5 − 1.</t>
-  </si>
-  <si>
-    <t>Normální aproximace</t>
-  </si>
-  <si>
     <t>Hranice počtu úspěchů</t>
   </si>
   <si>
@@ -300,7 +297,7 @@
     <t>Stres</t>
   </si>
   <si>
-    <t>Pohoda</t>
+    <t>Bez vysokého stresu</t>
   </si>
   <si>
     <t>Žena</t>
@@ -336,7 +333,7 @@
     <t>Výklad: přirozené četnosti, úplná pravděpodobnost, Bayesova věta, dvě prevalence</t>
   </si>
   <si>
-    <t>Modelové hodnoty zvolené pro výklad. Nejde o vlastnosti skutečného dotazníku ani o skutečný výskyt poruchy. Hotový výpočet je na listu Bayes.</t>
+    <t>Modelové hodnoty zvolené pro výklad. Nejde o vlastnosti skutečného dotazníku ani o skutečný výskyt poruchy. Při srovnání skupin předpokládáme stejnou senzitivitu a specificitu. Hotový výpočet je na listu Bayes.</t>
   </si>
   <si>
     <t>Počet otázek krátkého testu</t>
@@ -462,7 +459,7 @@
     <t>Cvičení 6</t>
   </si>
   <si>
-    <t>Modelové hodnoty. Nejde o vlastnosti skutečného dotazníku.</t>
+    <t>Modelové hodnoty. Nejde o vlastnosti skutečného dotazníku. Při obou prevalencích předpokládáme stejnou senzitivitu a specificitu.</t>
   </si>
   <si>
     <t>Podíl zelených taxíků</t>
@@ -477,7 +474,7 @@
     <t>Cvičení 7</t>
   </si>
   <si>
-    <t>Čísla podle Howella (2013, s. 122–123), který uvádí úlohu Tverského a Kahnemana; znění zadání je upraveno.</t>
+    <t>Čísla podle Howella (2013, s. 122–123), který uvádí úlohu Tverského a Kahnemana; znění zadání je upraveno. Předpokládáme stejnou pravděpodobnost účasti na nehodě pro každý taxík.</t>
   </si>
   <si>
     <t>Počet vybavených slov</t>
@@ -643,6 +640,9 @@
   </si>
   <si>
     <t>Pravděpodobnosti a modelové četnosti nejsou záznamy o jednotlivých lidech.</t>
+  </si>
+  <si>
+    <t>B4: 0 až 20; B5: 1 až 20 (celá čísla).</t>
   </si>
 </sst>
 </file>
@@ -732,7 +732,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="33">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -761,16 +761,13 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="1" fontId="1" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="165" fontId="1" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="2" fontId="1" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="1" fontId="1" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="1" fontId="1" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="166" fontId="1" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
@@ -796,6 +793,42 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyProtection="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="1" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="1" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="1" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="1" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="1" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="1" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center"/>
+      <protection locked="0"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1130,7 +1163,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D0F6EF17-C69F-477C-AE36-E3352F7C5F8B}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{504294FE-A6BC-4EC0-A5E1-DE36AAA572D4}">
   <dimension ref="A1:C31"/>
   <sheetFormatPr defaultRowHeight="14.3" x14ac:dyDescent="0.25"/>
   <cols>
@@ -1139,11 +1172,11 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" ht="30.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="21" t="s">
-        <v>152</v>
-      </c>
-      <c r="B1" s="19"/>
-      <c r="C1" s="19"/>
+      <c r="A1" s="20" t="s">
+        <v>151</v>
+      </c>
+      <c r="B1" s="18"/>
+      <c r="C1" s="18"/>
     </row>
     <row r="2" spans="1:3" ht="30.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="1"/>
@@ -1151,75 +1184,75 @@
       <c r="C2" s="1"/>
     </row>
     <row r="3" spans="1:3" ht="30.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="20" t="s">
+      <c r="A3" s="19" t="s">
+        <v>152</v>
+      </c>
+      <c r="B3" s="18"/>
+      <c r="C3" s="18"/>
+    </row>
+    <row r="4" spans="1:3" ht="30.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="19" t="s">
         <v>153</v>
       </c>
-      <c r="B3" s="19"/>
-      <c r="C3" s="19"/>
-    </row>
-    <row r="4" spans="1:3" ht="30.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="20" t="s">
-        <v>154</v>
-      </c>
-      <c r="B4" s="19"/>
-      <c r="C4" s="19"/>
+      <c r="B4" s="18"/>
+      <c r="C4" s="18"/>
     </row>
     <row r="5" spans="1:3" ht="30.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="20" t="s">
+      <c r="A5" s="19" t="s">
+        <v>193</v>
+      </c>
+      <c r="B5" s="18"/>
+      <c r="C5" s="18"/>
+    </row>
+    <row r="6" spans="1:3" ht="30.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="19" t="s">
         <v>194</v>
       </c>
-      <c r="B5" s="19"/>
-      <c r="C5" s="19"/>
-    </row>
-    <row r="6" spans="1:3" ht="30.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="20" t="s">
-        <v>195</v>
-      </c>
-      <c r="B6" s="19"/>
-      <c r="C6" s="19"/>
+      <c r="B6" s="18"/>
+      <c r="C6" s="18"/>
     </row>
     <row r="7" spans="1:3" ht="30.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
+        <v>154</v>
+      </c>
+      <c r="B7" s="3" t="s">
         <v>155</v>
       </c>
-      <c r="B7" s="3" t="s">
+      <c r="C7" s="3" t="s">
         <v>156</v>
-      </c>
-      <c r="C7" s="3" t="s">
-        <v>157</v>
       </c>
     </row>
     <row r="8" spans="1:3" ht="30.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
+        <v>157</v>
+      </c>
+      <c r="B8" s="2" t="s">
         <v>158</v>
       </c>
-      <c r="B8" s="2" t="s">
-        <v>159</v>
-      </c>
       <c r="C8" s="2" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
     </row>
     <row r="9" spans="1:3" ht="30.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
+        <v>159</v>
+      </c>
+      <c r="B9" s="2" t="s">
         <v>160</v>
       </c>
-      <c r="B9" s="2" t="s">
-        <v>161</v>
-      </c>
       <c r="C9" s="2" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="10" spans="1:3" ht="30.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
     </row>
     <row r="11" spans="1:3" ht="30.1" customHeight="1" x14ac:dyDescent="0.25">
@@ -1227,197 +1260,197 @@
         <v>0</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
     </row>
     <row r="12" spans="1:3" ht="30.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
     </row>
     <row r="13" spans="1:3" ht="30.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
+        <v>164</v>
+      </c>
+      <c r="B13" s="2" t="s">
         <v>165</v>
       </c>
-      <c r="B13" s="2" t="s">
-        <v>166</v>
-      </c>
       <c r="C13" s="2" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
     </row>
     <row r="14" spans="1:3" ht="30.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
     </row>
     <row r="15" spans="1:3" ht="30.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
+        <v>167</v>
+      </c>
+      <c r="B15" s="2" t="s">
         <v>168</v>
       </c>
-      <c r="B15" s="2" t="s">
-        <v>169</v>
-      </c>
       <c r="C15" s="2" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
     </row>
     <row r="16" spans="1:3" ht="30.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
+        <v>169</v>
+      </c>
+      <c r="B16" s="2" t="s">
         <v>170</v>
       </c>
-      <c r="B16" s="2" t="s">
-        <v>171</v>
-      </c>
       <c r="C16" s="2" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
     </row>
     <row r="17" spans="1:3" ht="30.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
     </row>
     <row r="18" spans="1:3" ht="30.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
     </row>
     <row r="19" spans="1:3" ht="30.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
+        <v>173</v>
+      </c>
+      <c r="B19" s="2" t="s">
         <v>174</v>
       </c>
-      <c r="B19" s="2" t="s">
-        <v>175</v>
-      </c>
       <c r="C19" s="2" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
     </row>
     <row r="20" spans="1:3" ht="30.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
     </row>
     <row r="21" spans="1:3" ht="30.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
+        <v>176</v>
+      </c>
+      <c r="B21" s="2" t="s">
         <v>177</v>
       </c>
-      <c r="B21" s="2" t="s">
-        <v>178</v>
-      </c>
       <c r="C21" s="2" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
     </row>
     <row r="22" spans="1:3" ht="30.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
     </row>
     <row r="23" spans="1:3" ht="30.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="2" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="24" spans="1:3" ht="30.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
     </row>
     <row r="25" spans="1:3" ht="30.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="2" t="s">
+        <v>181</v>
+      </c>
+      <c r="B25" s="2" t="s">
         <v>182</v>
       </c>
-      <c r="B25" s="2" t="s">
+      <c r="C25" s="2" t="s">
         <v>183</v>
-      </c>
-      <c r="C25" s="2" t="s">
-        <v>184</v>
       </c>
     </row>
     <row r="26" spans="1:3" ht="30.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="2" t="s">
+        <v>184</v>
+      </c>
+      <c r="B26" s="2" t="s">
         <v>185</v>
       </c>
-      <c r="B26" s="2" t="s">
+      <c r="C26" s="2" t="s">
         <v>186</v>
-      </c>
-      <c r="C26" s="2" t="s">
-        <v>187</v>
       </c>
     </row>
     <row r="27" spans="1:3" ht="30.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="2" t="s">
+        <v>187</v>
+      </c>
+      <c r="B27" s="2" t="s">
         <v>188</v>
       </c>
-      <c r="B27" s="2" t="s">
+      <c r="C27" s="2" t="s">
         <v>189</v>
-      </c>
-      <c r="C27" s="2" t="s">
-        <v>190</v>
       </c>
     </row>
     <row r="28" spans="1:3" ht="30.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="2" t="s">
+        <v>190</v>
+      </c>
+      <c r="B28" s="2" t="s">
         <v>191</v>
       </c>
-      <c r="B28" s="2" t="s">
+      <c r="C28" s="2" t="s">
         <v>192</v>
-      </c>
-      <c r="C28" s="2" t="s">
-        <v>193</v>
       </c>
     </row>
     <row r="29" spans="1:3" ht="30.1" customHeight="1" x14ac:dyDescent="0.25">
@@ -1448,7 +1481,7 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9E327118-9EA2-41A7-9E8C-7332AE1B9E00}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{33C9804A-2502-4315-830F-BD505D699F9C}">
   <dimension ref="A1:D7"/>
   <sheetFormatPr defaultRowHeight="14.3" x14ac:dyDescent="0.25"/>
   <cols>
@@ -1459,72 +1492,72 @@
   <sheetData>
     <row r="1" spans="1:4" ht="46.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="B1" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="16" t="s">
-        <v>76</v>
+      <c r="D1" s="15" t="s">
+        <v>75</v>
       </c>
     </row>
     <row r="2" spans="1:4" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="15" t="s">
+      <c r="A2" s="14" t="s">
+        <v>93</v>
+      </c>
+      <c r="B2" s="14">
+        <v>5</v>
+      </c>
+      <c r="D2" s="17" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="14" t="s">
         <v>94</v>
       </c>
-      <c r="B2" s="15">
+      <c r="B3" s="14">
+        <v>4</v>
+      </c>
+      <c r="D3" s="16"/>
+    </row>
+    <row r="4" spans="1:4" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="14" t="s">
+        <v>95</v>
+      </c>
+      <c r="B4" s="14">
+        <v>0.25</v>
+      </c>
+      <c r="D4" s="17" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="14" t="s">
+        <v>96</v>
+      </c>
+      <c r="B5" s="14">
+        <v>20</v>
+      </c>
+      <c r="D5" s="16"/>
+    </row>
+    <row r="6" spans="1:4" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="14" t="s">
+        <v>47</v>
+      </c>
+      <c r="B6" s="14">
         <v>5</v>
       </c>
-      <c r="D2" s="18" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="15" t="s">
-        <v>95</v>
-      </c>
-      <c r="B3" s="15">
-        <v>4</v>
-      </c>
-      <c r="D3" s="17"/>
-    </row>
-    <row r="4" spans="1:4" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="15" t="s">
-        <v>96</v>
-      </c>
-      <c r="B4" s="15">
-        <v>0.25</v>
-      </c>
-      <c r="D4" s="18" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="15" t="s">
-        <v>97</v>
-      </c>
-      <c r="B5" s="15">
-        <v>20</v>
-      </c>
-      <c r="D5" s="17"/>
-    </row>
-    <row r="6" spans="1:4" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="15" t="s">
-        <v>46</v>
-      </c>
-      <c r="B6" s="15">
-        <v>5</v>
-      </c>
-      <c r="D6" s="17"/>
+      <c r="D6" s="16"/>
     </row>
     <row r="7" spans="1:4" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="15" t="s">
-        <v>47</v>
-      </c>
-      <c r="B7" s="15">
+      <c r="A7" s="14" t="s">
+        <v>48</v>
+      </c>
+      <c r="B7" s="14">
         <v>10</v>
       </c>
-      <c r="D7" s="17"/>
+      <c r="D7" s="16"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -1536,7 +1569,7 @@
 </file>
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B49852BA-8822-4B9A-AA77-38F63278489B}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2FC3EC76-D459-423E-B18A-1DA8D0924F2D}">
   <dimension ref="A1:C41"/>
   <sheetFormatPr defaultRowHeight="14.3" x14ac:dyDescent="0.25"/>
   <cols>
@@ -1546,219 +1579,219 @@
   <sheetData>
     <row r="1" spans="1:3" ht="46.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
+        <v>99</v>
+      </c>
+      <c r="C1" s="15" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="14">
+        <v>2</v>
+      </c>
+      <c r="C2" s="17" t="s">
         <v>100</v>
       </c>
-      <c r="C1" s="16" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="15">
+    </row>
+    <row r="3" spans="1:3" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="14">
+        <v>1</v>
+      </c>
+      <c r="C3" s="16"/>
+    </row>
+    <row r="4" spans="1:3" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="14">
         <v>2</v>
       </c>
-      <c r="C2" s="18" t="s">
+      <c r="C4" s="17" t="s">
         <v>101</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="15">
+    <row r="5" spans="1:3" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="14">
+        <v>3</v>
+      </c>
+      <c r="C5" s="16"/>
+    </row>
+    <row r="6" spans="1:3" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="14">
         <v>1</v>
       </c>
-      <c r="C3" s="17"/>
-    </row>
-    <row r="4" spans="1:3" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="15">
+      <c r="C6" s="16"/>
+    </row>
+    <row r="7" spans="1:3" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="14">
+        <v>0</v>
+      </c>
+      <c r="C7" s="16"/>
+    </row>
+    <row r="8" spans="1:3" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="14">
         <v>2</v>
       </c>
-      <c r="C4" s="18" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="15">
+    </row>
+    <row r="9" spans="1:3" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="14">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="14">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="14">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="14">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="14">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="14">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="14">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="14">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="17" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="14">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="14">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="14">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="20" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="14">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="21" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="14">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="14">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A23" s="14">
         <v>3</v>
       </c>
-      <c r="C5" s="17"/>
-    </row>
-    <row r="6" spans="1:3" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="15">
+    </row>
+    <row r="24" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="14">
         <v>1</v>
       </c>
-      <c r="C6" s="17"/>
-    </row>
-    <row r="7" spans="1:3" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="15">
+    </row>
+    <row r="25" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A25" s="14">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="26" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A26" s="14">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="27" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A27" s="14">
         <v>0</v>
       </c>
-      <c r="C7" s="17"/>
-    </row>
-    <row r="8" spans="1:3" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="15">
+    </row>
+    <row r="28" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A28" s="14">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A29" s="14">
         <v>2</v>
       </c>
     </row>
-    <row r="9" spans="1:3" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="15">
+    <row r="30" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A30" s="14">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="31" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A31" s="14">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="32" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A32" s="14">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A33" s="14">
         <v>2</v>
       </c>
     </row>
-    <row r="10" spans="1:3" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="15">
+    <row r="34" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A34" s="14">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="35" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A35" s="14">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="36" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A36" s="14">
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:3" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="15">
+    <row r="37" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A37" s="14">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="38" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A38" s="14">
         <v>2</v>
       </c>
     </row>
-    <row r="12" spans="1:3" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="15">
+    <row r="39" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A39" s="14">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="40" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A40" s="14">
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="1:3" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="15">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="15">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="15" spans="1:3" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="15">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="16" spans="1:3" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="15">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="17" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="15">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="18" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="15">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="19" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="15">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="20" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="15">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="21" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="15">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="22" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="15">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="23" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="15">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="24" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="15">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="25" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="15">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="26" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="15">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="27" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="15">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="28" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="15">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="29" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="15">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="30" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="15">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="31" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="15">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="32" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="15">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="33" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="15">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="34" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="15">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="35" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="15">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="36" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A36" s="15">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="37" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A37" s="15">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="38" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A38" s="15">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="39" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A39" s="15">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="40" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A40" s="15">
-        <v>1</v>
-      </c>
-    </row>
     <row r="41" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A41" s="15">
+      <c r="A41" s="14">
         <v>0</v>
       </c>
     </row>
@@ -1772,7 +1805,7 @@
 </file>
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A1D4F0F4-EC3C-410F-84CD-7E0400989CDB}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{73135203-20D4-4997-B6D3-F5A286083494}">
   <dimension ref="A1:D7"/>
   <sheetFormatPr defaultRowHeight="14.3" x14ac:dyDescent="0.25"/>
   <cols>
@@ -1783,54 +1816,54 @@
   <sheetData>
     <row r="1" spans="1:4" ht="46.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="B1" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="16" t="s">
-        <v>76</v>
+      <c r="D1" s="15" t="s">
+        <v>75</v>
       </c>
     </row>
     <row r="2" spans="1:4" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="15" t="s">
+      <c r="A2" s="14" t="s">
+        <v>102</v>
+      </c>
+      <c r="B2" s="14">
+        <v>200</v>
+      </c>
+      <c r="D2" s="17" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="14" t="s">
         <v>103</v>
       </c>
-      <c r="B2" s="15">
-        <v>200</v>
-      </c>
-      <c r="D2" s="18" t="s">
+      <c r="B3" s="14">
+        <v>0.6</v>
+      </c>
+      <c r="D3" s="16"/>
+    </row>
+    <row r="4" spans="1:4" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="14" t="s">
+        <v>104</v>
+      </c>
+      <c r="B4" s="14">
+        <v>135</v>
+      </c>
+      <c r="D4" s="17" t="s">
         <v>106</v>
       </c>
     </row>
-    <row r="3" spans="1:4" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="15" t="s">
-        <v>104</v>
-      </c>
-      <c r="B3" s="15">
-        <v>0.6</v>
-      </c>
-      <c r="D3" s="17"/>
-    </row>
-    <row r="4" spans="1:4" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="15" t="s">
-        <v>105</v>
-      </c>
-      <c r="B4" s="15">
-        <v>135</v>
-      </c>
-      <c r="D4" s="18" t="s">
-        <v>107</v>
-      </c>
-    </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D5" s="17"/>
+      <c r="D5" s="16"/>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D6" s="17"/>
+      <c r="D6" s="16"/>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D7" s="17"/>
+      <c r="D7" s="16"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -1842,7 +1875,7 @@
 </file>
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A16010E6-9801-407F-982B-0FCC5436B97C}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{65ED7635-780A-4D6F-865E-7B52231A0F52}">
   <dimension ref="A1:D7"/>
   <sheetFormatPr defaultRowHeight="14.3" x14ac:dyDescent="0.25"/>
   <cols>
@@ -1852,48 +1885,48 @@
   <sheetData>
     <row r="1" spans="1:4" ht="46.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="B1" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="16" t="s">
-        <v>76</v>
+      <c r="D1" s="15" t="s">
+        <v>75</v>
       </c>
     </row>
     <row r="2" spans="1:4" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="15" t="s">
+      <c r="A2" s="14" t="s">
+        <v>107</v>
+      </c>
+      <c r="B2" s="14">
+        <v>100</v>
+      </c>
+      <c r="D2" s="17" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="14" t="s">
         <v>108</v>
       </c>
-      <c r="B2" s="15">
-        <v>100</v>
-      </c>
-      <c r="D2" s="18" t="s">
+      <c r="B3" s="14">
+        <v>3</v>
+      </c>
+      <c r="D3" s="16"/>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D4" s="17" t="s">
         <v>110</v>
       </c>
     </row>
-    <row r="3" spans="1:4" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="15" t="s">
-        <v>109</v>
-      </c>
-      <c r="B3" s="15">
-        <v>3</v>
-      </c>
-      <c r="D3" s="17"/>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D4" s="18" t="s">
-        <v>111</v>
-      </c>
-    </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D5" s="17"/>
+      <c r="D5" s="16"/>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D6" s="17"/>
+      <c r="D6" s="16"/>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D7" s="17"/>
+      <c r="D7" s="16"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -1905,7 +1938,7 @@
 </file>
 
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E6E1538D-96D4-491C-BB64-4F1305E6B691}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8F413F00-DC6A-4CB2-9255-C7992C253A15}">
   <dimension ref="A1:D7"/>
   <sheetFormatPr defaultRowHeight="14.3" x14ac:dyDescent="0.25"/>
   <cols>
@@ -1915,60 +1948,60 @@
   <sheetData>
     <row r="1" spans="1:4" ht="46.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
+        <v>111</v>
+      </c>
+      <c r="B1" s="4" t="s">
         <v>112</v>
       </c>
-      <c r="B1" s="4" t="s">
+      <c r="D1" s="15" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="14" t="s">
         <v>113</v>
       </c>
-      <c r="D1" s="16" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="15" t="s">
+      <c r="B2" s="14">
+        <v>24</v>
+      </c>
+      <c r="D2" s="17" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="14" t="s">
         <v>114</v>
       </c>
-      <c r="B2" s="15">
-        <v>24</v>
-      </c>
-      <c r="D2" s="18" t="s">
+      <c r="B3" s="14">
+        <v>18</v>
+      </c>
+      <c r="D3" s="16"/>
+    </row>
+    <row r="4" spans="1:4" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="14" t="s">
+        <v>115</v>
+      </c>
+      <c r="B4" s="14">
+        <v>12</v>
+      </c>
+      <c r="D4" s="17" t="s">
         <v>118</v>
       </c>
     </row>
-    <row r="3" spans="1:4" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="15" t="s">
-        <v>115</v>
-      </c>
-      <c r="B3" s="15">
-        <v>18</v>
-      </c>
-      <c r="D3" s="17"/>
-    </row>
-    <row r="4" spans="1:4" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="15" t="s">
+    <row r="5" spans="1:4" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="14" t="s">
         <v>116</v>
       </c>
-      <c r="B4" s="15">
-        <v>12</v>
-      </c>
-      <c r="D4" s="18" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="15" t="s">
-        <v>117</v>
-      </c>
-      <c r="B5" s="15">
+      <c r="B5" s="14">
         <v>6</v>
       </c>
-      <c r="D5" s="17"/>
+      <c r="D5" s="16"/>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D6" s="17"/>
+      <c r="D6" s="16"/>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D7" s="17"/>
+      <c r="D7" s="16"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -1980,7 +2013,7 @@
 </file>
 
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A09802A0-45B7-435A-AE00-F026207B7B23}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CC19B642-32B2-48BF-9718-6A76B5A5F690}">
   <dimension ref="A1:E7"/>
   <sheetFormatPr defaultRowHeight="14.3" x14ac:dyDescent="0.25"/>
   <cols>
@@ -1990,57 +2023,57 @@
   <sheetData>
     <row r="1" spans="1:5" ht="46.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
+        <v>119</v>
+      </c>
+      <c r="B1" s="4" t="s">
         <v>120</v>
       </c>
-      <c r="B1" s="4" t="s">
+      <c r="C1" s="4" t="s">
         <v>121</v>
       </c>
-      <c r="C1" s="4" t="s">
+      <c r="E1" s="15" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="14" t="s">
         <v>122</v>
       </c>
-      <c r="E1" s="16" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="15" t="s">
+      <c r="B2" s="14">
+        <v>54</v>
+      </c>
+      <c r="C2" s="14">
+        <v>26</v>
+      </c>
+      <c r="E2" s="17" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="14" t="s">
         <v>123</v>
       </c>
-      <c r="B2" s="15">
-        <v>54</v>
-      </c>
-      <c r="C2" s="15">
-        <v>26</v>
-      </c>
-      <c r="E2" s="18" t="s">
+      <c r="B3" s="14">
+        <v>27</v>
+      </c>
+      <c r="C3" s="14">
+        <v>43</v>
+      </c>
+      <c r="E3" s="16"/>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="E4" s="17" t="s">
         <v>125</v>
       </c>
     </row>
-    <row r="3" spans="1:5" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="15" t="s">
-        <v>124</v>
-      </c>
-      <c r="B3" s="15">
-        <v>27</v>
-      </c>
-      <c r="C3" s="15">
-        <v>43</v>
-      </c>
-      <c r="E3" s="17"/>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="E4" s="18" t="s">
-        <v>126</v>
-      </c>
-    </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="E5" s="17"/>
+      <c r="E5" s="16"/>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="E6" s="17"/>
+      <c r="E6" s="16"/>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="E7" s="17"/>
+      <c r="E7" s="16"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -2052,7 +2085,7 @@
 </file>
 
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B9CBC292-AB2B-438A-8B2D-4C7EA7D6C624}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A4FBAC73-1179-4421-BEB1-A967E6810CA5}">
   <dimension ref="A1:D7"/>
   <sheetFormatPr defaultRowHeight="14.3" x14ac:dyDescent="0.25"/>
   <cols>
@@ -2063,60 +2096,60 @@
   <sheetData>
     <row r="1" spans="1:4" ht="46.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="B1" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="16" t="s">
-        <v>76</v>
+      <c r="D1" s="15" t="s">
+        <v>75</v>
       </c>
     </row>
     <row r="2" spans="1:4" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="15" t="s">
-        <v>95</v>
-      </c>
-      <c r="B2" s="15">
+      <c r="A2" s="14" t="s">
+        <v>94</v>
+      </c>
+      <c r="B2" s="14">
         <v>4</v>
       </c>
-      <c r="D2" s="18" t="s">
+      <c r="D2" s="17" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="14" t="s">
+        <v>126</v>
+      </c>
+      <c r="B3" s="14">
+        <v>2</v>
+      </c>
+      <c r="D3" s="16"/>
+    </row>
+    <row r="4" spans="1:4" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="14" t="s">
+        <v>127</v>
+      </c>
+      <c r="B4" s="14">
+        <v>10</v>
+      </c>
+      <c r="D4" s="17" t="s">
         <v>130</v>
       </c>
     </row>
-    <row r="3" spans="1:4" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="15" t="s">
-        <v>127</v>
-      </c>
-      <c r="B3" s="15">
-        <v>2</v>
-      </c>
-      <c r="D3" s="17"/>
-    </row>
-    <row r="4" spans="1:4" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="15" t="s">
+    <row r="5" spans="1:4" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="14" t="s">
         <v>128</v>
       </c>
-      <c r="B4" s="15">
-        <v>10</v>
-      </c>
-      <c r="D4" s="18" t="s">
-        <v>131</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="15" t="s">
-        <v>129</v>
-      </c>
-      <c r="B5" s="15">
+      <c r="B5" s="14">
         <v>4</v>
       </c>
-      <c r="D5" s="17"/>
+      <c r="D5" s="16"/>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D6" s="17"/>
+      <c r="D6" s="16"/>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D7" s="17"/>
+      <c r="D7" s="16"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -2128,7 +2161,7 @@
 </file>
 
 <file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{742DD14A-1827-43F4-8D10-2943B4E470BA}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D163A58A-DADD-4406-BA6D-44F4B949CB32}">
   <dimension ref="A1:D7"/>
   <sheetFormatPr defaultRowHeight="14.3" x14ac:dyDescent="0.25"/>
   <cols>
@@ -2139,66 +2172,66 @@
   <sheetData>
     <row r="1" spans="1:4" ht="46.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="B1" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="16" t="s">
-        <v>76</v>
+      <c r="D1" s="15" t="s">
+        <v>75</v>
       </c>
     </row>
     <row r="2" spans="1:4" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="15" t="s">
+      <c r="A2" s="14" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="15">
+      <c r="B2" s="14">
         <v>1000</v>
       </c>
-      <c r="D2" s="18" t="s">
+      <c r="D2" s="17" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="14" t="s">
+        <v>4</v>
+      </c>
+      <c r="B3" s="14">
+        <v>0.8</v>
+      </c>
+      <c r="D3" s="16"/>
+    </row>
+    <row r="4" spans="1:4" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="14" t="s">
+        <v>5</v>
+      </c>
+      <c r="B4" s="14">
+        <v>0.9</v>
+      </c>
+      <c r="D4" s="17" t="s">
         <v>134</v>
       </c>
     </row>
-    <row r="3" spans="1:4" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="15" t="s">
-        <v>4</v>
-      </c>
-      <c r="B3" s="15">
-        <v>0.8</v>
-      </c>
-      <c r="D3" s="17"/>
-    </row>
-    <row r="4" spans="1:4" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="15" t="s">
-        <v>5</v>
-      </c>
-      <c r="B4" s="15">
-        <v>0.9</v>
-      </c>
-      <c r="D4" s="18" t="s">
-        <v>135</v>
-      </c>
-    </row>
     <row r="5" spans="1:4" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="15" t="s">
+      <c r="A5" s="14" t="s">
+        <v>131</v>
+      </c>
+      <c r="B5" s="14">
+        <v>0.05</v>
+      </c>
+      <c r="D5" s="16"/>
+    </row>
+    <row r="6" spans="1:4" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="14" t="s">
         <v>132</v>
       </c>
-      <c r="B5" s="15">
-        <v>0.05</v>
-      </c>
-      <c r="D5" s="17"/>
-    </row>
-    <row r="6" spans="1:4" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="15" t="s">
-        <v>133</v>
-      </c>
-      <c r="B6" s="15">
+      <c r="B6" s="14">
         <v>0.2</v>
       </c>
-      <c r="D6" s="17"/>
+      <c r="D6" s="16"/>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D7" s="17"/>
+      <c r="D7" s="16"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -2210,7 +2243,7 @@
 </file>
 
 <file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{93B02B4F-18CF-4E40-B272-02CD8B78B9BD}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{32583CC8-F49A-44B7-BB2E-E94C6EDB2F95}">
   <dimension ref="A1:D7"/>
   <sheetFormatPr defaultRowHeight="14.3" x14ac:dyDescent="0.25"/>
   <cols>
@@ -2221,54 +2254,54 @@
   <sheetData>
     <row r="1" spans="1:4" ht="46.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="B1" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="16" t="s">
-        <v>76</v>
+      <c r="D1" s="15" t="s">
+        <v>75</v>
       </c>
     </row>
     <row r="2" spans="1:4" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="15" t="s">
+      <c r="A2" s="14" t="s">
+        <v>135</v>
+      </c>
+      <c r="B2" s="14">
+        <v>0.85</v>
+      </c>
+      <c r="D2" s="17" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="14" t="s">
         <v>136</v>
       </c>
-      <c r="B2" s="15">
-        <v>0.85</v>
-      </c>
-      <c r="D2" s="18" t="s">
+      <c r="B3" s="14">
+        <v>0.15</v>
+      </c>
+      <c r="D3" s="16"/>
+    </row>
+    <row r="4" spans="1:4" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="14" t="s">
+        <v>137</v>
+      </c>
+      <c r="B4" s="14">
+        <v>0.8</v>
+      </c>
+      <c r="D4" s="17" t="s">
         <v>139</v>
       </c>
     </row>
-    <row r="3" spans="1:4" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="15" t="s">
-        <v>137</v>
-      </c>
-      <c r="B3" s="15">
-        <v>0.15</v>
-      </c>
-      <c r="D3" s="17"/>
-    </row>
-    <row r="4" spans="1:4" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="15" t="s">
-        <v>138</v>
-      </c>
-      <c r="B4" s="15">
-        <v>0.8</v>
-      </c>
-      <c r="D4" s="18" t="s">
-        <v>140</v>
-      </c>
-    </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D5" s="17"/>
+      <c r="D5" s="16"/>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D6" s="17"/>
+      <c r="D6" s="16"/>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D7" s="17"/>
+      <c r="D7" s="16"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -2280,7 +2313,7 @@
 </file>
 
 <file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3BBEBF62-EF3B-4F8C-BA7A-8EA32AD8381C}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{50C5A92C-CEAD-4A6C-9141-133B9297C723}">
   <dimension ref="A1:E7"/>
   <sheetFormatPr defaultRowHeight="14.3" x14ac:dyDescent="0.25"/>
   <cols>
@@ -2290,75 +2323,75 @@
   <sheetData>
     <row r="1" spans="1:5" ht="46.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
+        <v>140</v>
+      </c>
+      <c r="B1" s="4" t="s">
         <v>141</v>
       </c>
-      <c r="B1" s="4" t="s">
+      <c r="C1" s="4" t="s">
         <v>142</v>
       </c>
-      <c r="C1" s="4" t="s">
+      <c r="E1" s="15" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="14">
+        <v>0</v>
+      </c>
+      <c r="B2" s="14">
+        <v>0.1</v>
+      </c>
+      <c r="C2" s="14">
+        <v>3</v>
+      </c>
+      <c r="E2" s="17" t="s">
         <v>143</v>
       </c>
-      <c r="E1" s="16" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="15">
-        <v>0</v>
-      </c>
-      <c r="B2" s="15">
-        <v>0.1</v>
-      </c>
-      <c r="C2" s="15">
+    </row>
+    <row r="3" spans="1:5" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="14">
+        <v>1</v>
+      </c>
+      <c r="B3" s="14">
+        <v>0.4</v>
+      </c>
+      <c r="C3" s="14">
+        <v>7</v>
+      </c>
+      <c r="E3" s="16"/>
+    </row>
+    <row r="4" spans="1:5" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="14">
+        <v>2</v>
+      </c>
+      <c r="B4" s="14">
+        <v>0.35</v>
+      </c>
+      <c r="C4" s="14">
+        <v>8</v>
+      </c>
+      <c r="E4" s="17" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="14">
         <v>3</v>
       </c>
-      <c r="E2" s="18" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="15">
-        <v>1</v>
-      </c>
-      <c r="B3" s="15">
-        <v>0.4</v>
-      </c>
-      <c r="C3" s="15">
-        <v>7</v>
-      </c>
-      <c r="E3" s="17"/>
-    </row>
-    <row r="4" spans="1:5" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="15">
+      <c r="B5" s="14">
+        <v>0.15</v>
+      </c>
+      <c r="C5" s="14">
         <v>2</v>
       </c>
-      <c r="B4" s="15">
-        <v>0.35</v>
-      </c>
-      <c r="C4" s="15">
-        <v>8</v>
-      </c>
-      <c r="E4" s="18" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="15">
-        <v>3</v>
-      </c>
-      <c r="B5" s="15">
-        <v>0.15</v>
-      </c>
-      <c r="C5" s="15">
-        <v>2</v>
-      </c>
-      <c r="E5" s="17"/>
+      <c r="E5" s="16"/>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="E6" s="17"/>
+      <c r="E6" s="16"/>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="E7" s="17"/>
+      <c r="E7" s="16"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -2370,7 +2403,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4300F14A-94F8-4C1E-9476-0BE1C3844366}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{67AACCD7-FBFE-492A-8F02-14A4258432D0}">
   <dimension ref="A1:F22"/>
   <sheetFormatPr defaultRowHeight="14.3" x14ac:dyDescent="0.25"/>
   <cols>
@@ -2658,7 +2691,7 @@
 </file>
 
 <file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{73E5AB1F-EB8D-4C08-913B-AD1A98B8E68F}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A47140AF-D867-4B4D-9595-738C8084B0DB}">
   <dimension ref="A1:D7"/>
   <sheetFormatPr defaultRowHeight="14.3" x14ac:dyDescent="0.25"/>
   <cols>
@@ -2669,54 +2702,54 @@
   <sheetData>
     <row r="1" spans="1:4" ht="46.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="B1" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="16" t="s">
-        <v>76</v>
+      <c r="D1" s="15" t="s">
+        <v>75</v>
       </c>
     </row>
     <row r="2" spans="1:4" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="15" t="s">
+      <c r="A2" s="14" t="s">
+        <v>145</v>
+      </c>
+      <c r="B2" s="14">
+        <v>4</v>
+      </c>
+      <c r="D2" s="17" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="14" t="s">
+        <v>95</v>
+      </c>
+      <c r="B3" s="14">
+        <v>0.5</v>
+      </c>
+      <c r="D3" s="16"/>
+    </row>
+    <row r="4" spans="1:4" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="14" t="s">
         <v>146</v>
       </c>
-      <c r="B2" s="15">
-        <v>4</v>
-      </c>
-      <c r="D2" s="18" t="s">
-        <v>148</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="15" t="s">
-        <v>96</v>
-      </c>
-      <c r="B3" s="15">
-        <v>0.5</v>
-      </c>
-      <c r="D3" s="17"/>
-    </row>
-    <row r="4" spans="1:4" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="15" t="s">
-        <v>147</v>
-      </c>
-      <c r="B4" s="15">
+      <c r="B4" s="14">
         <v>3</v>
       </c>
-      <c r="D4" s="18" t="s">
-        <v>131</v>
+      <c r="D4" s="17" t="s">
+        <v>130</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D5" s="17"/>
+      <c r="D5" s="16"/>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D6" s="17"/>
+      <c r="D6" s="16"/>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D7" s="17"/>
+      <c r="D7" s="16"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -2728,7 +2761,7 @@
 </file>
 
 <file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C97D83DC-8C83-4463-8EE0-4F9AE08333E6}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6D942BE7-B90A-4F38-90DC-3C53CBEF6A12}">
   <dimension ref="A1:D7"/>
   <sheetFormatPr defaultRowHeight="14.3" x14ac:dyDescent="0.25"/>
   <cols>
@@ -2739,60 +2772,60 @@
   <sheetData>
     <row r="1" spans="1:4" ht="46.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="B1" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="16" t="s">
-        <v>76</v>
+      <c r="D1" s="15" t="s">
+        <v>75</v>
       </c>
     </row>
     <row r="2" spans="1:4" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="15" t="s">
-        <v>146</v>
-      </c>
-      <c r="B2" s="15">
+      <c r="A2" s="14" t="s">
+        <v>145</v>
+      </c>
+      <c r="B2" s="14">
         <v>15</v>
       </c>
-      <c r="D2" s="18" t="s">
-        <v>149</v>
+      <c r="D2" s="17" t="s">
+        <v>148</v>
       </c>
     </row>
     <row r="3" spans="1:4" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="15" t="s">
-        <v>95</v>
-      </c>
-      <c r="B3" s="15">
+      <c r="A3" s="14" t="s">
+        <v>94</v>
+      </c>
+      <c r="B3" s="14">
         <v>5</v>
       </c>
-      <c r="D3" s="17"/>
+      <c r="D3" s="16"/>
     </row>
     <row r="4" spans="1:4" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="15" t="s">
-        <v>46</v>
-      </c>
-      <c r="B4" s="15">
+      <c r="A4" s="14" t="s">
+        <v>47</v>
+      </c>
+      <c r="B4" s="14">
         <v>3</v>
       </c>
-      <c r="D4" s="18" t="s">
-        <v>131</v>
+      <c r="D4" s="17" t="s">
+        <v>130</v>
       </c>
     </row>
     <row r="5" spans="1:4" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="15" t="s">
-        <v>47</v>
-      </c>
-      <c r="B5" s="15">
+      <c r="A5" s="14" t="s">
+        <v>48</v>
+      </c>
+      <c r="B5" s="14">
         <v>7</v>
       </c>
-      <c r="D5" s="17"/>
+      <c r="D5" s="16"/>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D6" s="17"/>
+      <c r="D6" s="16"/>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D7" s="17"/>
+      <c r="D7" s="16"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -2804,7 +2837,7 @@
 </file>
 
 <file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B1725C09-B1DF-4BB8-B36A-4C11DFB0EBB6}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9A93A5D7-FB07-4516-A2DD-ED6A02A068D0}">
   <dimension ref="A1:D7"/>
   <sheetFormatPr defaultRowHeight="14.3" x14ac:dyDescent="0.25"/>
   <cols>
@@ -2815,54 +2848,54 @@
   <sheetData>
     <row r="1" spans="1:4" ht="46.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="B1" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="16" t="s">
-        <v>76</v>
+      <c r="D1" s="15" t="s">
+        <v>75</v>
       </c>
     </row>
     <row r="2" spans="1:4" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="15" t="s">
-        <v>146</v>
-      </c>
-      <c r="B2" s="15">
+      <c r="A2" s="14" t="s">
+        <v>145</v>
+      </c>
+      <c r="B2" s="14">
         <v>100</v>
       </c>
-      <c r="D2" s="18" t="s">
+      <c r="D2" s="17" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="14" t="s">
+        <v>95</v>
+      </c>
+      <c r="B3" s="14">
+        <v>0.5</v>
+      </c>
+      <c r="D3" s="16"/>
+    </row>
+    <row r="4" spans="1:4" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="14" t="s">
+        <v>104</v>
+      </c>
+      <c r="B4" s="14">
+        <v>65</v>
+      </c>
+      <c r="D4" s="17" t="s">
         <v>150</v>
       </c>
     </row>
-    <row r="3" spans="1:4" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="15" t="s">
-        <v>96</v>
-      </c>
-      <c r="B3" s="15">
-        <v>0.5</v>
-      </c>
-      <c r="D3" s="17"/>
-    </row>
-    <row r="4" spans="1:4" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="15" t="s">
-        <v>105</v>
-      </c>
-      <c r="B4" s="15">
-        <v>65</v>
-      </c>
-      <c r="D4" s="18" t="s">
-        <v>151</v>
-      </c>
-    </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D5" s="17"/>
+      <c r="D5" s="16"/>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D6" s="17"/>
+      <c r="D6" s="16"/>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D7" s="17"/>
+      <c r="D7" s="16"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -2874,690 +2907,720 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5A915078-AB32-4DB1-BDD0-8A42E11D13A4}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F26D0604-64F3-4919-8A4A-4707090C36F7}">
   <dimension ref="A1:F22"/>
   <sheetFormatPr defaultRowHeight="14.3" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="34.625" customWidth="1"/>
-    <col min="2" max="4" width="14.625" customWidth="1"/>
-    <col min="5" max="5" width="3.625" customWidth="1"/>
-    <col min="6" max="6" width="52.625" customWidth="1"/>
+    <col min="1" max="1" width="34.625" style="23" customWidth="1"/>
+    <col min="2" max="4" width="14.625" style="23" customWidth="1"/>
+    <col min="5" max="5" width="3.625" style="23" customWidth="1"/>
+    <col min="6" max="6" width="60.625" style="23" customWidth="1"/>
+    <col min="7" max="16384" width="9" style="23"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="34" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="4" t="s">
+      <c r="A1" s="21" t="s">
         <v>26</v>
       </c>
-      <c r="B1" s="4" t="s">
+      <c r="B1" s="21" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1"/>
-      <c r="F1" s="1"/>
+      <c r="C1" s="22"/>
+      <c r="D1" s="22"/>
+      <c r="E1" s="22"/>
+      <c r="F1" s="22"/>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A2" s="2" t="s">
+      <c r="A2" s="24" t="s">
         <v>27</v>
       </c>
-      <c r="B2" s="10">
+      <c r="B2" s="22">
         <v>5</v>
       </c>
-      <c r="C2" s="1"/>
-      <c r="D2" s="1"/>
-      <c r="E2" s="1"/>
-      <c r="F2" s="9" t="s">
+      <c r="C2" s="22"/>
+      <c r="D2" s="22"/>
+      <c r="E2" s="22"/>
+      <c r="F2" s="25" t="s">
         <v>39</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A3" s="2" t="s">
+      <c r="A3" s="24" t="s">
         <v>28</v>
       </c>
-      <c r="B3" s="6">
+      <c r="B3" s="30">
         <v>0.25</v>
       </c>
-      <c r="C3" s="1"/>
-      <c r="D3" s="1"/>
-      <c r="E3" s="1"/>
-      <c r="F3" s="9" t="s">
+      <c r="C3" s="22"/>
+      <c r="D3" s="22"/>
+      <c r="E3" s="22"/>
+      <c r="F3" s="25" t="s">
         <v>40</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A4" s="1"/>
-      <c r="B4" s="1"/>
-      <c r="C4" s="1"/>
-      <c r="D4" s="1"/>
-      <c r="E4" s="1"/>
-      <c r="F4" s="1"/>
+      <c r="A4" s="22"/>
+      <c r="B4" s="22"/>
+      <c r="C4" s="22"/>
+      <c r="D4" s="22"/>
+      <c r="E4" s="22"/>
+      <c r="F4" s="22"/>
     </row>
     <row r="5" spans="1:6" ht="34" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="4" t="s">
+      <c r="A5" s="21" t="s">
         <v>29</v>
       </c>
-      <c r="B5" s="4" t="s">
+      <c r="B5" s="21" t="s">
         <v>30</v>
       </c>
-      <c r="C5" s="4" t="s">
+      <c r="C5" s="21" t="s">
         <v>31</v>
       </c>
-      <c r="D5" s="4" t="s">
+      <c r="D5" s="21" t="s">
         <v>32</v>
       </c>
-      <c r="E5" s="1"/>
-      <c r="F5" s="9" t="s">
-        <v>20</v>
+      <c r="E5" s="22"/>
+      <c r="F5" s="25" t="s">
+        <v>41</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A6" s="10">
+      <c r="A6" s="22">
         <v>0</v>
       </c>
-      <c r="B6" s="11">
-        <f>_xlfn.BINOM.DIST(A6,$B$2,$B$3,FALSE)</f>
-        <v>0.23730468750000006</v>
-      </c>
-      <c r="C6" s="11">
+      <c r="B6" s="26">
+        <f>(1-$B$3)^$B$2</f>
+        <v>0.2373046875</v>
+      </c>
+      <c r="C6" s="26">
         <f>_xlfn.BINOM.DIST(A6,$B$2,$B$3,TRUE)</f>
         <v>0.23730468750000006</v>
       </c>
-      <c r="D6" s="11">
+      <c r="D6" s="26">
         <f>1-C6+B6</f>
         <v>1</v>
       </c>
-      <c r="E6" s="1"/>
-      <c r="F6" s="1"/>
+      <c r="E6" s="22"/>
+      <c r="F6" s="22"/>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A7" s="10">
+      <c r="A7" s="22">
         <v>1</v>
       </c>
-      <c r="B7" s="11">
+      <c r="B7" s="26">
         <f>_xlfn.BINOM.DIST(A7,$B$2,$B$3,FALSE)</f>
         <v>0.3955078125</v>
       </c>
-      <c r="C7" s="11">
+      <c r="C7" s="26">
         <f>_xlfn.BINOM.DIST(A7,$B$2,$B$3,TRUE)</f>
         <v>0.6328125</v>
       </c>
-      <c r="D7" s="11">
+      <c r="D7" s="26">
         <f>1-C7+B7</f>
         <v>0.7626953125</v>
       </c>
-      <c r="E7" s="1"/>
-      <c r="F7" s="9" t="s">
-        <v>41</v>
+      <c r="E7" s="22"/>
+      <c r="F7" s="25" t="s">
+        <v>42</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A8" s="10">
+      <c r="A8" s="22">
         <v>2</v>
       </c>
-      <c r="B8" s="11">
+      <c r="B8" s="26">
         <f>_xlfn.BINOM.DIST(A8,$B$2,$B$3,FALSE)</f>
         <v>0.26367187499999994</v>
       </c>
-      <c r="C8" s="11">
+      <c r="C8" s="26">
         <f>_xlfn.BINOM.DIST(A8,$B$2,$B$3,TRUE)</f>
         <v>0.896484375</v>
       </c>
-      <c r="D8" s="11">
+      <c r="D8" s="26">
         <f>1-C8+B8</f>
         <v>0.36718749999999994</v>
       </c>
-      <c r="E8" s="1"/>
-      <c r="F8" s="1"/>
+      <c r="E8" s="22"/>
+      <c r="F8" s="22"/>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A9" s="10">
+      <c r="A9" s="22">
         <v>3</v>
       </c>
-      <c r="B9" s="11">
+      <c r="B9" s="26">
         <f>_xlfn.BINOM.DIST(A9,$B$2,$B$3,FALSE)</f>
         <v>8.7890625000000042E-2</v>
       </c>
-      <c r="C9" s="11">
+      <c r="C9" s="26">
         <f>_xlfn.BINOM.DIST(A9,$B$2,$B$3,TRUE)</f>
         <v>0.984375</v>
       </c>
-      <c r="D9" s="11">
+      <c r="D9" s="26">
         <f>1-C9+B9</f>
         <v>0.10351562500000004</v>
       </c>
-      <c r="E9" s="1"/>
-      <c r="F9" s="1"/>
+      <c r="E9" s="22"/>
+      <c r="F9" s="22"/>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A10" s="10">
+      <c r="A10" s="22">
         <v>4</v>
       </c>
-      <c r="B10" s="11">
+      <c r="B10" s="26">
         <f>_xlfn.BINOM.DIST(A10,$B$2,$B$3,FALSE)</f>
         <v>1.4648437500000005E-2</v>
       </c>
-      <c r="C10" s="11">
+      <c r="C10" s="26">
         <f>_xlfn.BINOM.DIST(A10,$B$2,$B$3,TRUE)</f>
         <v>0.9990234375</v>
       </c>
-      <c r="D10" s="11">
+      <c r="D10" s="26">
         <f>1-C10+B10</f>
         <v>1.5625000000000007E-2</v>
       </c>
-      <c r="E10" s="1"/>
-      <c r="F10" s="1"/>
+      <c r="E10" s="22"/>
+      <c r="F10" s="22"/>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A11" s="10">
+      <c r="A11" s="22">
         <v>5</v>
       </c>
-      <c r="B11" s="11">
+      <c r="B11" s="26">
         <f>_xlfn.BINOM.DIST(A11,$B$2,$B$3,FALSE)</f>
         <v>9.765625E-4</v>
       </c>
-      <c r="C11" s="11">
+      <c r="C11" s="26">
         <f>_xlfn.BINOM.DIST(A11,$B$2,$B$3,TRUE)</f>
         <v>1</v>
       </c>
-      <c r="D11" s="11">
+      <c r="D11" s="26">
         <f>1-C11+B11</f>
         <v>9.765625E-4</v>
       </c>
-      <c r="E11" s="1"/>
-      <c r="F11" s="1"/>
+      <c r="E11" s="22"/>
+      <c r="F11" s="22"/>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A12" s="1"/>
-      <c r="B12" s="1"/>
-      <c r="C12" s="1"/>
-      <c r="D12" s="1"/>
-      <c r="E12" s="1"/>
-      <c r="F12" s="1"/>
+      <c r="A12" s="22"/>
+      <c r="B12" s="22"/>
+      <c r="C12" s="22"/>
+      <c r="D12" s="22"/>
+      <c r="E12" s="22"/>
+      <c r="F12" s="22"/>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A13" s="2" t="s">
+      <c r="A13" s="24" t="s">
         <v>33</v>
       </c>
-      <c r="B13" s="11">
+      <c r="B13" s="26">
         <f>SUM(B6:B11)</f>
         <v>1</v>
       </c>
-      <c r="C13" s="1"/>
-      <c r="D13" s="1"/>
-      <c r="E13" s="1"/>
-      <c r="F13" s="9" t="s">
-        <v>42</v>
+      <c r="C13" s="22"/>
+      <c r="D13" s="22"/>
+      <c r="E13" s="22"/>
+      <c r="F13" s="25" t="s">
+        <v>43</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A14" s="2" t="s">
+      <c r="A14" s="24" t="s">
         <v>34</v>
       </c>
-      <c r="B14" s="12">
+      <c r="B14" s="27">
         <f>B2*B3</f>
         <v>1.25</v>
       </c>
-      <c r="C14" s="1"/>
-      <c r="D14" s="1"/>
-      <c r="E14" s="1"/>
-      <c r="F14" s="1"/>
+      <c r="C14" s="22"/>
+      <c r="D14" s="22"/>
+      <c r="E14" s="22"/>
+      <c r="F14" s="22"/>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A15" s="2" t="s">
+      <c r="A15" s="24" t="s">
         <v>35</v>
       </c>
-      <c r="B15" s="8">
+      <c r="B15" s="28">
         <f>SQRT(B2*B3*(1-B3))</f>
         <v>0.96824583655185426</v>
       </c>
-      <c r="C15" s="1"/>
-      <c r="D15" s="1"/>
-      <c r="E15" s="1"/>
-      <c r="F15" s="1"/>
+      <c r="C15" s="22"/>
+      <c r="D15" s="22"/>
+      <c r="E15" s="22"/>
+      <c r="F15" s="22"/>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A16" s="1"/>
-      <c r="B16" s="1"/>
-      <c r="C16" s="1"/>
-      <c r="D16" s="1"/>
-      <c r="E16" s="1"/>
-      <c r="F16" s="1"/>
+      <c r="A16" s="22"/>
+      <c r="B16" s="22"/>
+      <c r="C16" s="22"/>
+      <c r="D16" s="22"/>
+      <c r="E16" s="22"/>
+      <c r="F16" s="22"/>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A17" s="2" t="s">
+      <c r="A17" s="24" t="s">
         <v>36</v>
       </c>
-      <c r="B17" s="13">
+      <c r="B17" s="29">
         <f>FACT(5)</f>
         <v>120</v>
       </c>
-      <c r="C17" s="1"/>
-      <c r="D17" s="1"/>
-      <c r="E17" s="1"/>
-      <c r="F17" s="1"/>
+      <c r="C17" s="22"/>
+      <c r="D17" s="22"/>
+      <c r="E17" s="22"/>
+      <c r="F17" s="22"/>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A18" s="2" t="s">
+      <c r="A18" s="24" t="s">
         <v>37</v>
       </c>
-      <c r="B18" s="13">
+      <c r="B18" s="29">
         <f>COMBIN(5,2)</f>
         <v>10</v>
       </c>
-      <c r="C18" s="1"/>
-      <c r="D18" s="1"/>
-      <c r="E18" s="1"/>
-      <c r="F18" s="1"/>
+      <c r="C18" s="22"/>
+      <c r="D18" s="22"/>
+      <c r="E18" s="22"/>
+      <c r="F18" s="22"/>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A19" s="2" t="s">
+      <c r="A19" s="24" t="s">
         <v>38</v>
       </c>
-      <c r="B19" s="11">
+      <c r="B19" s="26">
         <f>B18*B3^2*(1-B3)^3</f>
         <v>0.263671875</v>
       </c>
-      <c r="C19" s="1"/>
-      <c r="D19" s="1"/>
-      <c r="E19" s="1"/>
-      <c r="F19" s="9" t="s">
-        <v>43</v>
+      <c r="C19" s="22"/>
+      <c r="D19" s="22"/>
+      <c r="E19" s="22"/>
+      <c r="F19" s="25" t="s">
+        <v>44</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A20" s="1"/>
-      <c r="B20" s="1"/>
-      <c r="C20" s="1"/>
-      <c r="D20" s="1"/>
-      <c r="E20" s="1"/>
-      <c r="F20" s="1"/>
+      <c r="A20" s="22"/>
+      <c r="B20" s="22"/>
+      <c r="C20" s="22"/>
+      <c r="D20" s="22"/>
+      <c r="E20" s="22"/>
+      <c r="F20" s="22"/>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A21" s="1"/>
-      <c r="B21" s="1"/>
-      <c r="C21" s="1"/>
-      <c r="D21" s="1"/>
-      <c r="E21" s="1"/>
-      <c r="F21" s="1"/>
+      <c r="A21" s="22"/>
+      <c r="B21" s="22"/>
+      <c r="C21" s="22"/>
+      <c r="D21" s="22"/>
+      <c r="E21" s="22"/>
+      <c r="F21" s="22"/>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A22" s="1"/>
-      <c r="B22" s="1"/>
-      <c r="C22" s="1"/>
-      <c r="D22" s="1"/>
-      <c r="E22" s="1"/>
-      <c r="F22" s="1"/>
+      <c r="A22" s="22"/>
+      <c r="B22" s="22"/>
+      <c r="C22" s="22"/>
+      <c r="D22" s="22"/>
+      <c r="E22" s="22"/>
+      <c r="F22" s="22"/>
     </row>
   </sheetData>
+  <sheetProtection sheet="1" objects="1" scenarios="1"/>
+  <dataValidations count="1">
+    <dataValidation type="decimal" showInputMessage="1" showErrorMessage="1" sqref="B3" xr:uid="{49CA1E92-D368-4C47-B5F6-A8303D4F2FC3}">
+      <formula1>0</formula1>
+      <formula2>1</formula2>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A08F7A72-0170-499C-96C4-717C22BEB5DA}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FC01F049-871D-4B03-BA8F-E42DDA0EAAD7}">
   <dimension ref="A1:F22"/>
   <sheetFormatPr defaultRowHeight="14.3" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="46.625" customWidth="1"/>
-    <col min="2" max="2" width="14.625" customWidth="1"/>
-    <col min="3" max="3" width="3.625" customWidth="1"/>
-    <col min="4" max="4" width="10.625" customWidth="1"/>
-    <col min="5" max="5" width="14.625" customWidth="1"/>
+    <col min="1" max="1" width="46.625" style="23" customWidth="1"/>
+    <col min="2" max="2" width="14.625" style="23" customWidth="1"/>
+    <col min="3" max="3" width="3.625" style="23" customWidth="1"/>
+    <col min="4" max="4" width="10.625" style="23" customWidth="1"/>
+    <col min="5" max="5" width="14.625" style="23" customWidth="1"/>
+    <col min="6" max="16384" width="9" style="23"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="34" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="4" t="s">
-        <v>44</v>
-      </c>
-      <c r="B1" s="4" t="s">
+      <c r="A1" s="21" t="s">
+        <v>45</v>
+      </c>
+      <c r="B1" s="21" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1"/>
-      <c r="D1" s="4" t="s">
-        <v>45</v>
-      </c>
-      <c r="E1" s="4" t="s">
+      <c r="C1" s="22"/>
+      <c r="D1" s="21" t="s">
+        <v>46</v>
+      </c>
+      <c r="E1" s="21" t="s">
         <v>30</v>
       </c>
-      <c r="F1" s="1"/>
+      <c r="F1" s="22"/>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A2" s="2" t="s">
+      <c r="A2" s="24" t="s">
         <v>27</v>
       </c>
-      <c r="B2" s="10">
+      <c r="B2" s="22">
         <v>20</v>
       </c>
-      <c r="C2" s="1"/>
-      <c r="D2" s="10">
+      <c r="C2" s="22"/>
+      <c r="D2" s="22">
         <v>0</v>
       </c>
-      <c r="E2" s="11">
-        <f>_xlfn.BINOM.DIST(D2,$B$2,$B$3,FALSE)</f>
-        <v>3.1712119389339963E-3</v>
-      </c>
-      <c r="F2" s="1"/>
+      <c r="E2" s="26">
+        <f>(1-$B$3)^$B$2</f>
+        <v>3.1712119389339932E-3</v>
+      </c>
+      <c r="F2" s="22"/>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A3" s="2" t="s">
+      <c r="A3" s="24" t="s">
         <v>28</v>
       </c>
-      <c r="B3" s="6">
+      <c r="B3" s="30">
         <v>0.25</v>
       </c>
-      <c r="C3" s="1"/>
-      <c r="D3" s="10">
+      <c r="C3" s="22"/>
+      <c r="D3" s="22">
         <v>1</v>
       </c>
-      <c r="E3" s="11">
+      <c r="E3" s="26">
         <f>_xlfn.BINOM.DIST(D3,$B$2,$B$3,FALSE)</f>
         <v>2.1141412926226615E-2</v>
       </c>
-      <c r="F3" s="1"/>
+      <c r="F3" s="22"/>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A4" s="2" t="s">
-        <v>46</v>
-      </c>
-      <c r="B4" s="10">
+      <c r="A4" s="24" t="s">
+        <v>47</v>
+      </c>
+      <c r="B4" s="32">
         <v>5</v>
       </c>
-      <c r="C4" s="1"/>
-      <c r="D4" s="10">
+      <c r="C4" s="22"/>
+      <c r="D4" s="22">
         <v>2</v>
       </c>
-      <c r="E4" s="11">
+      <c r="E4" s="26">
         <f>_xlfn.BINOM.DIST(D4,$B$2,$B$3,FALSE)</f>
         <v>6.6947807599717662E-2</v>
       </c>
-      <c r="F4" s="1"/>
+      <c r="F4" s="22"/>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A5" s="2" t="s">
-        <v>47</v>
-      </c>
-      <c r="B5" s="10">
+      <c r="A5" s="24" t="s">
+        <v>48</v>
+      </c>
+      <c r="B5" s="32">
         <v>10</v>
       </c>
-      <c r="C5" s="1"/>
-      <c r="D5" s="10">
+      <c r="C5" s="22"/>
+      <c r="D5" s="22">
         <v>3</v>
       </c>
-      <c r="E5" s="11">
+      <c r="E5" s="26">
         <f>_xlfn.BINOM.DIST(D5,$B$2,$B$3,FALSE)</f>
         <v>0.13389561519943524</v>
       </c>
-      <c r="F5" s="1"/>
+      <c r="F5" s="22"/>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A6" s="1"/>
-      <c r="B6" s="1"/>
-      <c r="C6" s="1"/>
-      <c r="D6" s="10">
+      <c r="A6" s="22"/>
+      <c r="B6" s="22"/>
+      <c r="C6" s="22"/>
+      <c r="D6" s="22">
         <v>4</v>
       </c>
-      <c r="E6" s="11">
+      <c r="E6" s="26">
         <f>_xlfn.BINOM.DIST(D6,$B$2,$B$3,FALSE)</f>
         <v>0.18968545486586663</v>
       </c>
-      <c r="F6" s="1"/>
+      <c r="F6" s="22"/>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A7" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="B7" s="11">
-        <f>_xlfn.BINOM.DIST(B4,B2,B3,FALSE)</f>
+      <c r="A7" s="22" t="str">
+        <f>"Právě: P(X = "&amp;B4&amp;")"</f>
+        <v>Právě: P(X = 5)</v>
+      </c>
+      <c r="B7" s="26">
+        <f>IF(B4=0,(1-B3)^B2,_xlfn.BINOM.DIST(B4,B2,B3,FALSE))</f>
         <v>0.20233115185692441</v>
       </c>
-      <c r="C7" s="1"/>
-      <c r="D7" s="10">
+      <c r="C7" s="22"/>
+      <c r="D7" s="22">
         <v>5</v>
       </c>
-      <c r="E7" s="11">
+      <c r="E7" s="26">
         <f>_xlfn.BINOM.DIST(D7,$B$2,$B$3,FALSE)</f>
         <v>0.20233115185692441</v>
       </c>
-      <c r="F7" s="1"/>
+      <c r="F7" s="22"/>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A8" s="2" t="s">
-        <v>49</v>
-      </c>
-      <c r="B8" s="11">
+      <c r="A8" s="22" t="str">
+        <f>"Nejvýše: P(X ≤ "&amp;B4&amp;")"</f>
+        <v>Nejvýše: P(X ≤ 5)</v>
+      </c>
+      <c r="B8" s="26">
         <f>_xlfn.BINOM.DIST(B4,B2,B3,TRUE)</f>
         <v>0.61717265438710467</v>
       </c>
-      <c r="C8" s="1"/>
-      <c r="D8" s="10">
+      <c r="C8" s="22"/>
+      <c r="D8" s="22">
         <v>6</v>
       </c>
-      <c r="E8" s="11">
+      <c r="E8" s="26">
         <f>_xlfn.BINOM.DIST(D8,$B$2,$B$3,FALSE)</f>
         <v>0.1686092932141037</v>
       </c>
-      <c r="F8" s="1"/>
+      <c r="F8" s="22"/>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A9" s="2" t="s">
-        <v>50</v>
-      </c>
-      <c r="B9" s="11">
+      <c r="A9" s="22" t="str">
+        <f>"Alespoň: P(X ≥ "&amp;B5&amp;")"</f>
+        <v>Alespoň: P(X ≥ 10)</v>
+      </c>
+      <c r="B9" s="26">
         <f>1-_xlfn.BINOM.DIST(B5-1,B2,B3,TRUE)</f>
         <v>1.3864416943761171E-2</v>
       </c>
-      <c r="C9" s="1"/>
-      <c r="D9" s="10">
+      <c r="C9" s="22"/>
+      <c r="D9" s="22">
         <v>7</v>
       </c>
-      <c r="E9" s="11">
+      <c r="E9" s="26">
         <f>_xlfn.BINOM.DIST(D9,$B$2,$B$3,FALSE)</f>
         <v>0.11240619547606913</v>
       </c>
-      <c r="F9" s="1"/>
+      <c r="F9" s="22"/>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A10" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="B10" s="11">
+      <c r="A10" s="24" t="s">
+        <v>49</v>
+      </c>
+      <c r="B10" s="26">
         <f>_xlfn.BINOM.DIST.RANGE(B2,B3,B5,B2)</f>
         <v>1.3864416943761178E-2</v>
       </c>
-      <c r="C10" s="1"/>
-      <c r="D10" s="10">
+      <c r="C10" s="22"/>
+      <c r="D10" s="22">
         <v>8</v>
       </c>
-      <c r="E10" s="11">
+      <c r="E10" s="26">
         <f>_xlfn.BINOM.DIST(D10,$B$2,$B$3,FALSE)</f>
         <v>6.0886689216204062E-2</v>
       </c>
-      <c r="F10" s="1"/>
+      <c r="F10" s="22"/>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A11" s="2" t="s">
+      <c r="A11" s="24" t="s">
         <v>34</v>
       </c>
-      <c r="B11" s="12">
+      <c r="B11" s="27">
         <f>B2*B3</f>
         <v>5</v>
       </c>
-      <c r="C11" s="1"/>
-      <c r="D11" s="10">
+      <c r="C11" s="22"/>
+      <c r="D11" s="22">
         <v>9</v>
       </c>
-      <c r="E11" s="11">
+      <c r="E11" s="26">
         <f>_xlfn.BINOM.DIST(D11,$B$2,$B$3,FALSE)</f>
         <v>2.7060750762757369E-2</v>
       </c>
-      <c r="F11" s="1"/>
+      <c r="F11" s="22"/>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A12" s="2" t="s">
+      <c r="A12" s="24" t="s">
         <v>35</v>
       </c>
-      <c r="B12" s="8">
+      <c r="B12" s="28">
         <f>SQRT(B2*B3*(1-B3))</f>
         <v>1.9364916731037085</v>
       </c>
-      <c r="C12" s="1"/>
-      <c r="D12" s="10">
+      <c r="C12" s="22"/>
+      <c r="D12" s="22">
         <v>10</v>
       </c>
-      <c r="E12" s="11">
+      <c r="E12" s="26">
         <f>_xlfn.BINOM.DIST(D12,$B$2,$B$3,FALSE)</f>
         <v>9.9222752796777041E-3</v>
       </c>
-      <c r="F12" s="1"/>
+      <c r="F12" s="22"/>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A13" s="2" t="s">
-        <v>52</v>
-      </c>
-      <c r="B13" s="13">
-        <f>_xlfn.BINOM.INV(B2,B3,0.95)</f>
+      <c r="A13" s="24" t="s">
+        <v>50</v>
+      </c>
+      <c r="B13" s="29">
+        <f>IF(B3=0,0,IF(B3=1,B2,_xlfn.BINOM.INV(B2,B3,0.95)))</f>
         <v>8</v>
       </c>
-      <c r="C13" s="1"/>
-      <c r="D13" s="10">
+      <c r="C13" s="22"/>
+      <c r="D13" s="22">
         <v>11</v>
       </c>
-      <c r="E13" s="11">
+      <c r="E13" s="26">
         <f>_xlfn.BINOM.DIST(D13,$B$2,$B$3,FALSE)</f>
         <v>3.0067500847508173E-3</v>
       </c>
-      <c r="F13" s="1"/>
+      <c r="F13" s="22"/>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A14" s="1"/>
-      <c r="B14" s="1"/>
-      <c r="C14" s="1"/>
-      <c r="D14" s="10">
+      <c r="A14" s="22"/>
+      <c r="B14" s="22"/>
+      <c r="C14" s="22"/>
+      <c r="D14" s="22">
         <v>12</v>
       </c>
-      <c r="E14" s="11">
+      <c r="E14" s="26">
         <f>_xlfn.BINOM.DIST(D14,$B$2,$B$3,FALSE)</f>
         <v>7.5168752118770586E-4</v>
       </c>
-      <c r="F14" s="1"/>
+      <c r="F14" s="22"/>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A15" s="1"/>
-      <c r="B15" s="1"/>
-      <c r="C15" s="1"/>
-      <c r="D15" s="10">
+      <c r="A15" s="22"/>
+      <c r="B15" s="22"/>
+      <c r="C15" s="22"/>
+      <c r="D15" s="22">
         <v>13</v>
       </c>
-      <c r="E15" s="11">
+      <c r="E15" s="26">
         <f>_xlfn.BINOM.DIST(D15,$B$2,$B$3,FALSE)</f>
         <v>1.541923120385034E-4</v>
       </c>
-      <c r="F15" s="1"/>
+      <c r="F15" s="22"/>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A16" s="9" t="s">
-        <v>20</v>
-      </c>
-      <c r="B16" s="1"/>
-      <c r="C16" s="1"/>
-      <c r="D16" s="10">
+      <c r="A16" s="25" t="s">
+        <v>51</v>
+      </c>
+      <c r="B16" s="22"/>
+      <c r="C16" s="22"/>
+      <c r="D16" s="22">
         <v>14</v>
       </c>
-      <c r="E16" s="11">
+      <c r="E16" s="26">
         <f>_xlfn.BINOM.DIST(D16,$B$2,$B$3,FALSE)</f>
         <v>2.5698718673083962E-5</v>
       </c>
-      <c r="F16" s="1"/>
+      <c r="F16" s="22"/>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A17" s="9" t="s">
-        <v>53</v>
-      </c>
-      <c r="B17" s="1"/>
-      <c r="C17" s="1"/>
-      <c r="D17" s="10">
+      <c r="A17" s="25" t="s">
+        <v>52</v>
+      </c>
+      <c r="B17" s="22"/>
+      <c r="C17" s="22"/>
+      <c r="D17" s="22">
         <v>15</v>
       </c>
-      <c r="E17" s="11">
+      <c r="E17" s="26">
         <f>_xlfn.BINOM.DIST(D17,$B$2,$B$3,FALSE)</f>
         <v>3.42649582307786E-6</v>
       </c>
-      <c r="F17" s="1"/>
+      <c r="F17" s="22"/>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A18" s="1"/>
-      <c r="B18" s="1"/>
-      <c r="C18" s="1"/>
-      <c r="D18" s="10">
+      <c r="A18" s="24" t="s">
+        <v>195</v>
+      </c>
+      <c r="B18" s="22"/>
+      <c r="C18" s="22"/>
+      <c r="D18" s="22">
         <v>16</v>
       </c>
-      <c r="E18" s="11">
+      <c r="E18" s="26">
         <f>_xlfn.BINOM.DIST(D18,$B$2,$B$3,FALSE)</f>
         <v>3.5692664823727645E-7</v>
       </c>
-      <c r="F18" s="1"/>
+      <c r="F18" s="22"/>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A19" s="9" t="s">
-        <v>54</v>
-      </c>
-      <c r="B19" s="1"/>
-      <c r="C19" s="1"/>
-      <c r="D19" s="10">
+      <c r="A19" s="31" t="str">
+        <f>"Alespoň "&amp;B5&amp;" = 1 − nejvýše "&amp;(B5-1)&amp;", proto B5 − 1."</f>
+        <v>Alespoň 10 = 1 − nejvýše 9, proto B5 − 1.</v>
+      </c>
+      <c r="B19" s="22"/>
+      <c r="C19" s="22"/>
+      <c r="D19" s="22">
         <v>17</v>
       </c>
-      <c r="E19" s="11">
+      <c r="E19" s="26">
         <f>_xlfn.BINOM.DIST(D19,$B$2,$B$3,FALSE)</f>
         <v>2.7994246920570738E-8</v>
       </c>
-      <c r="F19" s="1"/>
+      <c r="F19" s="22"/>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A20" s="1"/>
-      <c r="B20" s="1"/>
-      <c r="C20" s="1"/>
-      <c r="D20" s="10">
+      <c r="A20" s="22"/>
+      <c r="B20" s="22"/>
+      <c r="C20" s="22"/>
+      <c r="D20" s="22">
         <v>18</v>
       </c>
-      <c r="E20" s="11">
+      <c r="E20" s="26">
         <f>_xlfn.BINOM.DIST(D20,$B$2,$B$3,FALSE)</f>
         <v>1.5552359400317114E-9</v>
       </c>
-      <c r="F20" s="1"/>
+      <c r="F20" s="22"/>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A21" s="1"/>
-      <c r="B21" s="1"/>
-      <c r="C21" s="1"/>
-      <c r="D21" s="10">
+      <c r="A21" s="22"/>
+      <c r="B21" s="22"/>
+      <c r="C21" s="22"/>
+      <c r="D21" s="22">
         <v>19</v>
       </c>
-      <c r="E21" s="11">
+      <c r="E21" s="26">
         <f>_xlfn.BINOM.DIST(D21,$B$2,$B$3,FALSE)</f>
         <v>5.4569682106375856E-11</v>
       </c>
-      <c r="F21" s="1"/>
+      <c r="F21" s="22"/>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A22" s="1"/>
-      <c r="B22" s="1"/>
-      <c r="C22" s="1"/>
-      <c r="D22" s="10">
+      <c r="A22" s="22"/>
+      <c r="B22" s="22"/>
+      <c r="C22" s="22"/>
+      <c r="D22" s="22">
         <v>20</v>
       </c>
-      <c r="E22" s="11">
+      <c r="E22" s="26">
         <f>_xlfn.BINOM.DIST(D22,$B$2,$B$3,FALSE)</f>
         <v>9.0949470177292824E-13</v>
       </c>
-      <c r="F22" s="1"/>
+      <c r="F22" s="22"/>
     </row>
   </sheetData>
+  <sheetProtection sheet="1" objects="1" scenarios="1"/>
+  <dataValidations count="3">
+    <dataValidation type="decimal" showInputMessage="1" showErrorMessage="1" sqref="B3" xr:uid="{32928621-6C2A-4E9C-8269-D6ECAECB7D20}">
+      <formula1>0</formula1>
+      <formula2>1</formula2>
+    </dataValidation>
+    <dataValidation type="whole" showInputMessage="1" showErrorMessage="1" sqref="B4" xr:uid="{EAD94F5B-BCC8-4560-BBCB-6AC27F591EB1}">
+      <formula1>0</formula1>
+      <formula2>20</formula2>
+    </dataValidation>
+    <dataValidation type="whole" showInputMessage="1" showErrorMessage="1" sqref="B5" xr:uid="{4EBDF847-92D1-47B6-84D2-CDBBF0E695AA}">
+      <formula1>1</formula1>
+      <formula2>20</formula2>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6779A5B5-A1C2-4FD5-9F79-6AFE306BB888}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6B06EAB7-68B9-41EC-846F-1809BCDB5789}">
   <dimension ref="A1:F22"/>
   <sheetFormatPr defaultRowHeight="14.3" x14ac:dyDescent="0.25"/>
   <cols>
@@ -3569,7 +3632,7 @@
   <sheetData>
     <row r="1" spans="1:6" ht="34" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="B1" s="4" t="s">
         <v>1</v>
@@ -3581,14 +3644,14 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="B2" s="10">
+        <v>54</v>
+      </c>
+      <c r="B2" s="12">
         <v>200</v>
       </c>
       <c r="C2" s="1"/>
       <c r="D2" s="9" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="E2" s="1"/>
       <c r="F2" s="1"/>
@@ -3607,9 +3670,9 @@
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>56</v>
-      </c>
-      <c r="B4" s="10">
+        <v>55</v>
+      </c>
+      <c r="B4" s="12">
         <v>135</v>
       </c>
       <c r="C4" s="1"/>
@@ -3629,24 +3692,24 @@
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>57</v>
-      </c>
-      <c r="B6" s="12">
+        <v>56</v>
+      </c>
+      <c r="B6" s="11">
         <f>B2*B3</f>
         <v>120</v>
       </c>
       <c r="C6" s="1"/>
       <c r="D6" s="9" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="E6" s="1"/>
       <c r="F6" s="1"/>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
-        <v>58</v>
-      </c>
-      <c r="B7" s="12">
+        <v>57</v>
+      </c>
+      <c r="B7" s="11">
         <f>B2*(1-B3)</f>
         <v>80</v>
       </c>
@@ -3670,7 +3733,7 @@
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B9" s="8">
         <f>(B4-B6)/B8</f>
@@ -3683,39 +3746,39 @@
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="B10" s="11">
+        <v>59</v>
+      </c>
+      <c r="B10" s="10">
         <f>1-_xlfn.NORM.S.DIST(B9,TRUE)</f>
         <v>1.51914109882888E-2</v>
       </c>
       <c r="C10" s="1"/>
       <c r="D10" s="9" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E10" s="1"/>
       <c r="F10" s="1"/>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
-        <v>61</v>
-      </c>
-      <c r="B11" s="11">
+        <v>60</v>
+      </c>
+      <c r="B11" s="10">
         <f>1-_xlfn.BINOM.DIST(B4-1,B2,B3,TRUE)</f>
         <v>1.7307341051347791E-2</v>
       </c>
       <c r="C11" s="1"/>
       <c r="D11" s="9" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="E11" s="1"/>
       <c r="F11" s="1"/>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
-        <v>62</v>
-      </c>
-      <c r="B12" s="11">
+        <v>61</v>
+      </c>
+      <c r="B12" s="10">
         <f>1-_xlfn.NORM.DIST(B4-0.5,B6,B8,TRUE)</f>
         <v>1.8179276586395288E-2</v>
       </c>
@@ -3734,7 +3797,7 @@
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B14" s="8">
         <f>B4/B2</f>
@@ -3747,9 +3810,9 @@
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
-        <v>64</v>
-      </c>
-      <c r="B15" s="14">
+        <v>63</v>
+      </c>
+      <c r="B15" s="13">
         <f>SQRT(B3*(1-B3)/B2)</f>
         <v>3.4641016151377546E-2</v>
       </c>
@@ -3760,7 +3823,7 @@
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B16" s="8">
         <f>(B14-B3)/B15</f>
@@ -3768,7 +3831,7 @@
       </c>
       <c r="C16" s="1"/>
       <c r="D16" s="9" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="E16" s="1"/>
       <c r="F16" s="1"/>
@@ -3827,7 +3890,7 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{257764B6-587A-470C-8FB3-19CE21906CB0}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E920D08C-9789-4727-8597-333196F0A8BF}">
   <dimension ref="A1:D7"/>
   <sheetFormatPr defaultRowHeight="14.3" x14ac:dyDescent="0.25"/>
   <cols>
@@ -3837,54 +3900,54 @@
   <sheetData>
     <row r="1" spans="1:4" ht="46.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
+        <v>70</v>
+      </c>
+      <c r="B1" s="4" t="s">
         <v>71</v>
       </c>
-      <c r="B1" s="4" t="s">
+      <c r="D1" s="15" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="14" t="s">
         <v>72</v>
       </c>
-      <c r="D1" s="16" t="s">
+      <c r="B2" s="14">
+        <v>40</v>
+      </c>
+      <c r="D2" s="17" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="2" spans="1:4" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="15" t="s">
+    <row r="3" spans="1:4" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="14" t="s">
         <v>73</v>
       </c>
-      <c r="B2" s="15">
-        <v>40</v>
-      </c>
-      <c r="D2" s="18" t="s">
+      <c r="B3" s="14">
+        <v>35</v>
+      </c>
+      <c r="D3" s="16"/>
+    </row>
+    <row r="4" spans="1:4" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="14" t="s">
+        <v>74</v>
+      </c>
+      <c r="B4" s="14">
+        <v>25</v>
+      </c>
+      <c r="D4" s="17" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="3" spans="1:4" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="15" t="s">
-        <v>74</v>
-      </c>
-      <c r="B3" s="15">
-        <v>35</v>
-      </c>
-      <c r="D3" s="17"/>
-    </row>
-    <row r="4" spans="1:4" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="15" t="s">
-        <v>75</v>
-      </c>
-      <c r="B4" s="15">
-        <v>25</v>
-      </c>
-      <c r="D4" s="18" t="s">
-        <v>78</v>
-      </c>
-    </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D5" s="17"/>
+      <c r="D5" s="16"/>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D6" s="17"/>
+      <c r="D6" s="16"/>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D7" s="17"/>
+      <c r="D7" s="16"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -3896,7 +3959,7 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9C8870F7-321C-499A-B39C-67D64A0C3712}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{888D1082-A2EE-4ED0-B885-83CF43D2EE06}">
   <dimension ref="A1:E7"/>
   <sheetFormatPr defaultRowHeight="14.3" x14ac:dyDescent="0.25"/>
   <cols>
@@ -3906,57 +3969,57 @@
   <sheetData>
     <row r="1" spans="1:5" ht="46.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
+        <v>78</v>
+      </c>
+      <c r="B1" s="4" t="s">
         <v>79</v>
       </c>
-      <c r="B1" s="4" t="s">
+      <c r="C1" s="4" t="s">
         <v>80</v>
       </c>
-      <c r="C1" s="4" t="s">
+      <c r="E1" s="15" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="14" t="s">
         <v>81</v>
       </c>
-      <c r="E1" s="16" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="15" t="s">
+      <c r="B2" s="14">
+        <v>40</v>
+      </c>
+      <c r="C2" s="14">
+        <v>60</v>
+      </c>
+      <c r="E2" s="17" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="14" t="s">
         <v>82</v>
       </c>
-      <c r="B2" s="15">
-        <v>40</v>
-      </c>
-      <c r="C2" s="15">
-        <v>60</v>
-      </c>
-      <c r="E2" s="18" t="s">
+      <c r="B3" s="14">
+        <v>30</v>
+      </c>
+      <c r="C3" s="14">
+        <v>70</v>
+      </c>
+      <c r="E3" s="16"/>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="E4" s="17" t="s">
         <v>84</v>
       </c>
     </row>
-    <row r="3" spans="1:5" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="15" t="s">
-        <v>83</v>
-      </c>
-      <c r="B3" s="15">
-        <v>30</v>
-      </c>
-      <c r="C3" s="15">
-        <v>70</v>
-      </c>
-      <c r="E3" s="17"/>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="E4" s="18" t="s">
-        <v>85</v>
-      </c>
-    </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="E5" s="17"/>
+      <c r="E5" s="16"/>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="E6" s="17"/>
+      <c r="E6" s="16"/>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="E7" s="17"/>
+      <c r="E7" s="16"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -3968,7 +4031,7 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{428B3A6F-D4FE-47FD-9E25-DC0E9B3A7E07}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{40684DF2-F235-4ACC-A664-CB41909FFB27}">
   <dimension ref="A1:E7"/>
   <sheetFormatPr defaultRowHeight="14.3" x14ac:dyDescent="0.25"/>
   <cols>
@@ -3978,57 +4041,57 @@
   <sheetData>
     <row r="1" spans="1:5" ht="46.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
+        <v>78</v>
+      </c>
+      <c r="B1" s="4" t="s">
         <v>79</v>
       </c>
-      <c r="B1" s="4" t="s">
+      <c r="C1" s="4" t="s">
         <v>80</v>
       </c>
-      <c r="C1" s="4" t="s">
+      <c r="E1" s="15" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="14" t="s">
         <v>81</v>
       </c>
-      <c r="E1" s="16" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="15" t="s">
+      <c r="B2" s="14">
+        <v>30</v>
+      </c>
+      <c r="C2" s="14">
+        <v>70</v>
+      </c>
+      <c r="E2" s="17" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="14" t="s">
         <v>82</v>
       </c>
-      <c r="B2" s="15">
+      <c r="B3" s="14">
         <v>30</v>
       </c>
-      <c r="C2" s="15">
+      <c r="C3" s="14">
         <v>70</v>
       </c>
-      <c r="E2" s="18" t="s">
+      <c r="E3" s="16"/>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="E4" s="17" t="s">
         <v>86</v>
       </c>
     </row>
-    <row r="3" spans="1:5" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="15" t="s">
-        <v>83</v>
-      </c>
-      <c r="B3" s="15">
-        <v>30</v>
-      </c>
-      <c r="C3" s="15">
-        <v>70</v>
-      </c>
-      <c r="E3" s="17"/>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="E4" s="18" t="s">
-        <v>87</v>
-      </c>
-    </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="E5" s="17"/>
+      <c r="E5" s="16"/>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="E6" s="17"/>
+      <c r="E6" s="16"/>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="E7" s="17"/>
+      <c r="E7" s="16"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -4040,7 +4103,7 @@
 </file>
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{68B1D094-92C7-421B-8ED5-20F1D2185A2C}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7062D485-4339-4824-AF33-B35988D9AA34}">
   <dimension ref="A1:D7"/>
   <sheetFormatPr defaultRowHeight="14.3" x14ac:dyDescent="0.25"/>
   <cols>
@@ -4051,72 +4114,72 @@
   <sheetData>
     <row r="1" spans="1:4" ht="46.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="B1" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="16" t="s">
-        <v>76</v>
+      <c r="D1" s="15" t="s">
+        <v>75</v>
       </c>
     </row>
     <row r="2" spans="1:4" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="15" t="s">
+      <c r="A2" s="14" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="15">
+      <c r="B2" s="14">
         <v>1000</v>
       </c>
-      <c r="D2" s="18" t="s">
+      <c r="D2" s="17" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="14" t="s">
+        <v>88</v>
+      </c>
+      <c r="B3" s="14">
+        <v>0.1</v>
+      </c>
+      <c r="D3" s="16"/>
+    </row>
+    <row r="4" spans="1:4" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="14" t="s">
+        <v>4</v>
+      </c>
+      <c r="B4" s="14">
+        <v>0.95</v>
+      </c>
+      <c r="D4" s="17" t="s">
         <v>92</v>
       </c>
     </row>
-    <row r="3" spans="1:4" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="15" t="s">
+    <row r="5" spans="1:4" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="14" t="s">
+        <v>5</v>
+      </c>
+      <c r="B5" s="14">
+        <v>0.9</v>
+      </c>
+      <c r="D5" s="16"/>
+    </row>
+    <row r="6" spans="1:4" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="14" t="s">
         <v>89</v>
       </c>
-      <c r="B3" s="15">
-        <v>0.1</v>
-      </c>
-      <c r="D3" s="17"/>
-    </row>
-    <row r="4" spans="1:4" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="15" t="s">
-        <v>4</v>
-      </c>
-      <c r="B4" s="15">
-        <v>0.95</v>
-      </c>
-      <c r="D4" s="18" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="15" t="s">
-        <v>5</v>
-      </c>
-      <c r="B5" s="15">
-        <v>0.9</v>
-      </c>
-      <c r="D5" s="17"/>
-    </row>
-    <row r="6" spans="1:4" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="15" t="s">
+      <c r="B6" s="14">
+        <v>0.01</v>
+      </c>
+      <c r="D6" s="16"/>
+    </row>
+    <row r="7" spans="1:4" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="14" t="s">
         <v>90</v>
       </c>
-      <c r="B6" s="15">
-        <v>0.01</v>
-      </c>
-      <c r="D6" s="17"/>
-    </row>
-    <row r="7" spans="1:4" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="15" t="s">
-        <v>91</v>
-      </c>
-      <c r="B7" s="15">
+      <c r="B7" s="14">
         <v>10000</v>
       </c>
-      <c r="D7" s="17"/>
+      <c r="D7" s="16"/>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>

<commit_message>
Kapitola 5: zapracování autorových připomínek
Zachovává a dokončuje autorovy redakční úpravy kapitoly 5 a zapracovává
25 připomínek: úvody „Tento oddíl…“, přesnější četnostní pojetí, odvození
součinového pravidla a nezávislosti po krocích, obrácený směr nezávislosti,
význam pozitivního a negativního výsledku, tabulku čtyř kombinací stavu
a výsledku, přesnější vymezení přirozených četností (nový zdroj
Gigerenzer a Hoffrage 1995), popisky větví stromu, kombinace po sloupcích,
odlišení náhodné proměnné od rozdělení a vazbu na výběrový prostor.

Terminologie podle R52: opačný jev (číslo 1 − P zůstává doplněk do jedné),
prediktivní hodnota pozitivního/negativního testu, zvýšený/nízký stres.
Navarro citován s rokem 2026 (doplněk R42). Upraveny grafy, sešit,
kontroly, slovníček, značení a autorská dokumentace.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/kapitola_05.xlsx
+++ b/data/kapitola_05.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="202300"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{A686227C-91E5-4FD3-8D6B-63257186C438}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{AC8F8E12-DAE1-44B8-85DD-70AE72F2AD61}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-109" yWindow="-109" windowWidth="34995" windowHeight="19060" xr2:uid="{99AC8C74-C027-4117-BBC3-80F61B39B3A4}"/>
+    <workbookView xWindow="-109" yWindow="-109" windowWidth="34995" windowHeight="19060" xr2:uid="{19390E2A-1601-4290-B9FE-D6C88C124BE9}"/>
   </bookViews>
   <sheets>
     <sheet name="Prehled" sheetId="1" r:id="rId1"/>
@@ -99,10 +99,10 @@
     <t>Negativní celkem</t>
   </si>
   <si>
-    <t>Pozitivní prediktivní hodnota</t>
-  </si>
-  <si>
-    <t>Negativní prediktivní hodnota</t>
+    <t>Prediktivní hodnota pozitivního testu</t>
+  </si>
+  <si>
+    <t>Prediktivní hodnota negativního testu</t>
   </si>
   <si>
     <t>Úplná pravděpodobnost pozitivního výsledku</t>
@@ -285,7 +285,7 @@
     <t>Použití a původ</t>
   </si>
   <si>
-    <t>Výklad: výsledek, jev, doplněk, výběr bez vracení</t>
+    <t>Výklad: výsledek, jev, opačný jev, výběr bez vracení</t>
   </si>
   <si>
     <t>Autorská modelová krabice 100 kartiček. Četnosti, nikoli záznamy o lidech.</t>
@@ -294,10 +294,10 @@
     <t>Pohlaví</t>
   </si>
   <si>
-    <t>Stres</t>
-  </si>
-  <si>
-    <t>Bez vysokého stresu</t>
+    <t>Zvýšený stres</t>
+  </si>
+  <si>
+    <t>Nízký stres</t>
   </si>
   <si>
     <t>Žena</t>
@@ -315,7 +315,7 @@
     <t>Výklad: nezávislé jevy</t>
   </si>
   <si>
-    <t>Druhý autorský modelový soubor 200 studentů se stejným podílem stresu v obou řádcích.</t>
+    <t>Druhý autorský modelový soubor 200 studentů se stejným podílem zvýšeného stresu v obou řádcích.</t>
   </si>
   <si>
     <t>Vstup</t>
@@ -1163,7 +1163,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{504294FE-A6BC-4EC0-A5E1-DE36AAA572D4}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B69E3591-195A-4385-8FAB-4032512721E1}">
   <dimension ref="A1:C31"/>
   <sheetFormatPr defaultRowHeight="14.3" x14ac:dyDescent="0.25"/>
   <cols>
@@ -1481,7 +1481,7 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{33C9804A-2502-4315-830F-BD505D699F9C}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F340B4BD-3F78-40D8-AADD-74FACDAF6BB6}">
   <dimension ref="A1:D7"/>
   <sheetFormatPr defaultRowHeight="14.3" x14ac:dyDescent="0.25"/>
   <cols>
@@ -1569,7 +1569,7 @@
 </file>
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2FC3EC76-D459-423E-B18A-1DA8D0924F2D}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{28306F6A-A92E-492F-86DB-F3D4EDE72808}">
   <dimension ref="A1:C41"/>
   <sheetFormatPr defaultRowHeight="14.3" x14ac:dyDescent="0.25"/>
   <cols>
@@ -1805,7 +1805,7 @@
 </file>
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{73135203-20D4-4997-B6D3-F5A286083494}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DA8623A9-DC5A-47D0-94A7-0B8CDCDE6DA2}">
   <dimension ref="A1:D7"/>
   <sheetFormatPr defaultRowHeight="14.3" x14ac:dyDescent="0.25"/>
   <cols>
@@ -1875,7 +1875,7 @@
 </file>
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{65ED7635-780A-4D6F-865E-7B52231A0F52}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2CF7B3AC-23F4-4757-A836-D3EBA1BEA242}">
   <dimension ref="A1:D7"/>
   <sheetFormatPr defaultRowHeight="14.3" x14ac:dyDescent="0.25"/>
   <cols>
@@ -1938,7 +1938,7 @@
 </file>
 
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8F413F00-DC6A-4CB2-9255-C7992C253A15}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D453F6A4-93CD-4257-AE7A-CC63D633AF99}">
   <dimension ref="A1:D7"/>
   <sheetFormatPr defaultRowHeight="14.3" x14ac:dyDescent="0.25"/>
   <cols>
@@ -2013,7 +2013,7 @@
 </file>
 
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CC19B642-32B2-48BF-9718-6A76B5A5F690}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FCC713A0-D922-4A92-A2FA-5C96181EA5C2}">
   <dimension ref="A1:E7"/>
   <sheetFormatPr defaultRowHeight="14.3" x14ac:dyDescent="0.25"/>
   <cols>
@@ -2085,7 +2085,7 @@
 </file>
 
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A4FBAC73-1179-4421-BEB1-A967E6810CA5}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6A46A704-90D5-43B1-88B2-4CEADAADF85D}">
   <dimension ref="A1:D7"/>
   <sheetFormatPr defaultRowHeight="14.3" x14ac:dyDescent="0.25"/>
   <cols>
@@ -2161,7 +2161,7 @@
 </file>
 
 <file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D163A58A-DADD-4406-BA6D-44F4B949CB32}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{739BB9FA-7C03-4361-8DE5-CCF0B534EA46}">
   <dimension ref="A1:D7"/>
   <sheetFormatPr defaultRowHeight="14.3" x14ac:dyDescent="0.25"/>
   <cols>
@@ -2243,7 +2243,7 @@
 </file>
 
 <file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{32583CC8-F49A-44B7-BB2E-E94C6EDB2F95}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{966440C4-5229-4EDF-9E06-406E2A696B09}">
   <dimension ref="A1:D7"/>
   <sheetFormatPr defaultRowHeight="14.3" x14ac:dyDescent="0.25"/>
   <cols>
@@ -2313,7 +2313,7 @@
 </file>
 
 <file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{50C5A92C-CEAD-4A6C-9141-133B9297C723}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{703C9278-2FE5-4104-BCD1-F865C6D24A00}">
   <dimension ref="A1:E7"/>
   <sheetFormatPr defaultRowHeight="14.3" x14ac:dyDescent="0.25"/>
   <cols>
@@ -2403,7 +2403,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{67AACCD7-FBFE-492A-8F02-14A4258432D0}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{919B68F4-FF9B-40C8-8711-1A720F9A2611}">
   <dimension ref="A1:F22"/>
   <sheetFormatPr defaultRowHeight="14.3" x14ac:dyDescent="0.25"/>
   <cols>
@@ -2691,7 +2691,7 @@
 </file>
 
 <file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A47140AF-D867-4B4D-9595-738C8084B0DB}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{52FB11B8-A403-45BF-938B-0BD073718FC1}">
   <dimension ref="A1:D7"/>
   <sheetFormatPr defaultRowHeight="14.3" x14ac:dyDescent="0.25"/>
   <cols>
@@ -2761,7 +2761,7 @@
 </file>
 
 <file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6D942BE7-B90A-4F38-90DC-3C53CBEF6A12}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6A1BBCCB-0D0C-49E4-A6FF-AFCEAA491FE9}">
   <dimension ref="A1:D7"/>
   <sheetFormatPr defaultRowHeight="14.3" x14ac:dyDescent="0.25"/>
   <cols>
@@ -2837,7 +2837,7 @@
 </file>
 
 <file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9A93A5D7-FB07-4516-A2DD-ED6A02A068D0}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D50110A6-9BF0-44FD-9DEB-0C2EB5462731}">
   <dimension ref="A1:D7"/>
   <sheetFormatPr defaultRowHeight="14.3" x14ac:dyDescent="0.25"/>
   <cols>
@@ -2907,7 +2907,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F26D0604-64F3-4919-8A4A-4707090C36F7}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6E51F824-BD43-4506-89F4-02A0D1D7BBFA}">
   <dimension ref="A1:F22"/>
   <sheetFormatPr defaultRowHeight="14.3" x14ac:dyDescent="0.25"/>
   <cols>
@@ -3225,7 +3225,7 @@
   </sheetData>
   <sheetProtection sheet="1" objects="1" scenarios="1"/>
   <dataValidations count="1">
-    <dataValidation type="decimal" showInputMessage="1" showErrorMessage="1" sqref="B3" xr:uid="{49CA1E92-D368-4C47-B5F6-A8303D4F2FC3}">
+    <dataValidation type="decimal" showInputMessage="1" showErrorMessage="1" sqref="B3" xr:uid="{41ABE34A-9872-4F56-A74D-0F51296F8141}">
       <formula1>0</formula1>
       <formula2>1</formula2>
     </dataValidation>
@@ -3235,7 +3235,7 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FC01F049-871D-4B03-BA8F-E42DDA0EAAD7}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{97A37A58-62AE-4F4B-B342-6192CD2E475E}">
   <dimension ref="A1:F22"/>
   <sheetFormatPr defaultRowHeight="14.3" x14ac:dyDescent="0.25"/>
   <cols>
@@ -3602,15 +3602,15 @@
   </sheetData>
   <sheetProtection sheet="1" objects="1" scenarios="1"/>
   <dataValidations count="3">
-    <dataValidation type="decimal" showInputMessage="1" showErrorMessage="1" sqref="B3" xr:uid="{32928621-6C2A-4E9C-8269-D6ECAECB7D20}">
+    <dataValidation type="decimal" showInputMessage="1" showErrorMessage="1" sqref="B3" xr:uid="{FE24D493-E113-4A1D-A6B5-05E983C8FDAF}">
       <formula1>0</formula1>
       <formula2>1</formula2>
     </dataValidation>
-    <dataValidation type="whole" showInputMessage="1" showErrorMessage="1" sqref="B4" xr:uid="{EAD94F5B-BCC8-4560-BBCB-6AC27F591EB1}">
+    <dataValidation type="whole" showInputMessage="1" showErrorMessage="1" sqref="B4" xr:uid="{8199B101-04C2-4D1A-9399-AF91FD6BD672}">
       <formula1>0</formula1>
       <formula2>20</formula2>
     </dataValidation>
-    <dataValidation type="whole" showInputMessage="1" showErrorMessage="1" sqref="B5" xr:uid="{4EBDF847-92D1-47B6-84D2-CDBBF0E695AA}">
+    <dataValidation type="whole" showInputMessage="1" showErrorMessage="1" sqref="B5" xr:uid="{783E4E20-D815-4BB7-8E60-4D477154F551}">
       <formula1>1</formula1>
       <formula2>20</formula2>
     </dataValidation>
@@ -3620,7 +3620,7 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6B06EAB7-68B9-41EC-846F-1809BCDB5789}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C3CAFD66-F197-4F48-9A99-4395B5CB929A}">
   <dimension ref="A1:F22"/>
   <sheetFormatPr defaultRowHeight="14.3" x14ac:dyDescent="0.25"/>
   <cols>
@@ -3890,7 +3890,7 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E920D08C-9789-4727-8597-333196F0A8BF}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{337E78F8-4ECA-4FA4-B828-C38AF1068286}">
   <dimension ref="A1:D7"/>
   <sheetFormatPr defaultRowHeight="14.3" x14ac:dyDescent="0.25"/>
   <cols>
@@ -3959,7 +3959,7 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{888D1082-A2EE-4ED0-B885-83CF43D2EE06}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6C4E4FB1-670A-49CD-8718-F11F70085CB9}">
   <dimension ref="A1:E7"/>
   <sheetFormatPr defaultRowHeight="14.3" x14ac:dyDescent="0.25"/>
   <cols>
@@ -4031,7 +4031,7 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{40684DF2-F235-4ACC-A664-CB41909FFB27}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8E15E308-1E43-47FB-9DB3-7A97F99DEE13}">
   <dimension ref="A1:E7"/>
   <sheetFormatPr defaultRowHeight="14.3" x14ac:dyDescent="0.25"/>
   <cols>
@@ -4103,7 +4103,7 @@
 </file>
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7062D485-4339-4824-AF33-B35988D9AA34}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{956971CC-5CBD-4D88-A212-9C0DC2961505}">
   <dimension ref="A1:D7"/>
   <sheetFormatPr defaultRowHeight="14.3" x14ac:dyDescent="0.25"/>
   <cols>

</xml_diff>